<commit_message>
feat: wrongRoomType constraint check for certain lab/act in correct room
</commit_message>
<xml_diff>
--- a/java/hello-world/src/main/java/org/acme/schooltimetabling/generated/temp.xlsx
+++ b/java/hello-world/src/main/java/org/acme/schooltimetabling/generated/temp.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="107">
   <si>
     <t>Instructor Name</t>
   </si>
@@ -39,21 +39,24 @@
     <t>csc202</t>
   </si>
   <si>
+    <t>301</t>
+  </si>
+  <si>
+    <t>MWF 08:00 - 09:00</t>
+  </si>
+  <si>
+    <t>MWF 09:00 - 10:00</t>
+  </si>
+  <si>
+    <t>Beard, Stephen Robert</t>
+  </si>
+  <si>
+    <t>csc430</t>
+  </si>
+  <si>
     <t>255</t>
   </si>
   <si>
-    <t>MWF 08:00 - 09:00</t>
-  </si>
-  <si>
-    <t>MWF 09:00 - 10:00</t>
-  </si>
-  <si>
-    <t>Beard, Stephen Robert</t>
-  </si>
-  <si>
-    <t>csc430</t>
-  </si>
-  <si>
     <t>TR 08:00 - 09:30</t>
   </si>
   <si>
@@ -111,136 +114,130 @@
     <t>csc357</t>
   </si>
   <si>
+    <t>csc474</t>
+  </si>
+  <si>
     <t>TR 12:00 - 13:30</t>
   </si>
   <si>
     <t>TR 13:30 - 15:00</t>
   </si>
   <si>
-    <t>csc474</t>
+    <t>Einakian, Sussan</t>
+  </si>
+  <si>
+    <t>csc101</t>
+  </si>
+  <si>
+    <t>MWF 13:00 - 14:00</t>
+  </si>
+  <si>
+    <t>Frishberg, Daniel</t>
+  </si>
+  <si>
+    <t>csc445</t>
+  </si>
+  <si>
+    <t>LECTURE_ONLY</t>
+  </si>
+  <si>
+    <t>MTWR 09:00 - 10:00</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Gonzalez Sanchez, Javier</t>
+  </si>
+  <si>
+    <t>csc570</t>
+  </si>
+  <si>
+    <t>MTWR 11:00 - 12:00</t>
+  </si>
+  <si>
+    <t>Grow, April Marie</t>
+  </si>
+  <si>
+    <t>csc378</t>
+  </si>
+  <si>
+    <t>Hristov, Borislav</t>
+  </si>
+  <si>
+    <t>csc448</t>
+  </si>
+  <si>
+    <t>MWF 17:00 - 18:00</t>
+  </si>
+  <si>
+    <t>Hsu, Silas</t>
+  </si>
+  <si>
+    <t>csc437</t>
+  </si>
+  <si>
+    <t>Jones, Brian Thomas</t>
+  </si>
+  <si>
+    <t>csc232</t>
+  </si>
+  <si>
+    <t>MW 13:00 - 14:00</t>
+  </si>
+  <si>
+    <t>MW 14:00 - 15:00</t>
+  </si>
+  <si>
+    <t>MTWR 10:00 - 11:00</t>
+  </si>
+  <si>
+    <t>MTWR 12:00 - 13:00</t>
+  </si>
+  <si>
+    <t>Kalathas, Paris</t>
+  </si>
+  <si>
+    <t>csc203</t>
+  </si>
+  <si>
+    <t>Kazerouni, Ayaan</t>
+  </si>
+  <si>
+    <t>csc477</t>
+  </si>
+  <si>
+    <t>Keen, Aaron</t>
+  </si>
+  <si>
+    <t>256</t>
+  </si>
+  <si>
+    <t>Khan, Fahim Hasan</t>
+  </si>
+  <si>
+    <t>csc471</t>
+  </si>
+  <si>
+    <t>MWF 18:00 - 19:00</t>
+  </si>
+  <si>
+    <t>Klingenberg, Bernhard J.</t>
+  </si>
+  <si>
+    <t>csc406</t>
+  </si>
+  <si>
+    <t>Kubiak, Kenneth E.</t>
+  </si>
+  <si>
+    <t>csc307</t>
   </si>
   <si>
     <t>TR 15:00 - 16:30</t>
   </si>
   <si>
-    <t>TR 16:30 - 18:00</t>
-  </si>
-  <si>
-    <t>Einakian, Sussan</t>
-  </si>
-  <si>
-    <t>csc101</t>
-  </si>
-  <si>
-    <t>MWF 13:00 - 14:00</t>
-  </si>
-  <si>
-    <t>256</t>
-  </si>
-  <si>
-    <t>Frishberg, Daniel</t>
-  </si>
-  <si>
-    <t>csc445</t>
-  </si>
-  <si>
-    <t>LECTURE_ONLY</t>
-  </si>
-  <si>
-    <t>MTWR 09:00 - 10:00</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Gonzalez Sanchez, Javier</t>
-  </si>
-  <si>
-    <t>csc570</t>
-  </si>
-  <si>
-    <t>MTWR 11:00 - 12:00</t>
-  </si>
-  <si>
-    <t>Grow, April Marie</t>
-  </si>
-  <si>
-    <t>csc378</t>
-  </si>
-  <si>
-    <t>Hristov, Borislav</t>
-  </si>
-  <si>
-    <t>csc448</t>
-  </si>
-  <si>
-    <t>MWF 17:00 - 18:00</t>
-  </si>
-  <si>
-    <t>Hsu, Silas</t>
-  </si>
-  <si>
-    <t>csc437</t>
-  </si>
-  <si>
-    <t>MWF 18:00 - 19:00</t>
-  </si>
-  <si>
-    <t>Jones, Brian Thomas</t>
-  </si>
-  <si>
-    <t>csc232</t>
-  </si>
-  <si>
-    <t>MW 18:00 - 19:00</t>
-  </si>
-  <si>
-    <t>MW 19:00 - 20:00</t>
-  </si>
-  <si>
-    <t>MTWR 10:00 - 11:00</t>
-  </si>
-  <si>
-    <t>MTWR 12:00 - 13:00</t>
-  </si>
-  <si>
-    <t>Kalathas, Paris</t>
-  </si>
-  <si>
-    <t>csc203</t>
-  </si>
-  <si>
-    <t>Kazerouni, Ayaan</t>
-  </si>
-  <si>
-    <t>csc477</t>
-  </si>
-  <si>
-    <t>Keen, Aaron</t>
-  </si>
-  <si>
-    <t>Khan, Fahim Hasan</t>
-  </si>
-  <si>
-    <t>csc471</t>
-  </si>
-  <si>
-    <t>TR 18:00 - 19:30</t>
-  </si>
-  <si>
-    <t>Klingenberg, Bernhard J.</t>
-  </si>
-  <si>
-    <t>csc406</t>
-  </si>
-  <si>
-    <t>Kubiak, Kenneth E.</t>
-  </si>
-  <si>
-    <t>csc307</t>
-  </si>
-  <si>
-    <t>301</t>
+    <t>257</t>
   </si>
   <si>
     <t>Lindqvist, Ulf Erik</t>
@@ -249,12 +246,18 @@
     <t>csc320</t>
   </si>
   <si>
+    <t>192-333</t>
+  </si>
+  <si>
     <t>Mukherjee, Joydeep</t>
   </si>
   <si>
     <t>csc410</t>
   </si>
   <si>
+    <t>302</t>
+  </si>
+  <si>
     <t>Nico, Phillip L.</t>
   </si>
   <si>
@@ -267,10 +270,10 @@
     <t>csc569</t>
   </si>
   <si>
-    <t>TR 18:30 - 20:00</t>
-  </si>
-  <si>
-    <t>TR 20:00 - 21:30</t>
+    <t>TR 16:00 - 17:30</t>
+  </si>
+  <si>
+    <t>TR 17:30 - 19:00</t>
   </si>
   <si>
     <t>Peterson, Zachary N.J.</t>
@@ -282,12 +285,12 @@
     <t>csc466</t>
   </si>
   <si>
-    <t>257</t>
-  </si>
-  <si>
     <t>Rathi, Anita</t>
   </si>
   <si>
+    <t>232A</t>
+  </si>
+  <si>
     <t>Rivera, Vanessa</t>
   </si>
   <si>
@@ -300,21 +303,12 @@
     <t>csc349</t>
   </si>
   <si>
-    <t>TR 16:00 - 17:30</t>
-  </si>
-  <si>
-    <t>TR 17:30 - 19:00</t>
-  </si>
-  <si>
     <t>Schmitt, Paul</t>
   </si>
   <si>
     <t>Siu, Christopher E.</t>
   </si>
   <si>
-    <t>MWF 19:00 - 20:00</t>
-  </si>
-  <si>
     <t>Stanchev, Lubomir Petrov</t>
   </si>
   <si>
@@ -334,9 +328,6 @@
   </si>
   <si>
     <t>csc321</t>
-  </si>
-  <si>
-    <t>302</t>
   </si>
   <si>
     <t>Zielke, Christopher Patrick</t>
@@ -449,38 +440,38 @@
         <v>1</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>10</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s" s="0">
         <v>12</v>
@@ -489,18 +480,18 @@
         <v>1</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>7</v>
@@ -512,27 +503,27 @@
         <v>8</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C7" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F7" t="s" s="0">
         <v>9</v>
@@ -540,50 +531,50 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C8" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C9" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C10" t="b" s="0">
         <v>1</v>
@@ -592,38 +583,38 @@
         <v>8</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>33</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B11" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="C11" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E11" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="C11" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D11" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="E11" t="s" s="0">
+      <c r="F11" t="s" s="0">
         <v>35</v>
-      </c>
-      <c r="F11" t="s" s="0">
-        <v>36</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B12" t="s" s="0">
         <v>37</v>
-      </c>
-      <c r="B12" t="s" s="0">
-        <v>38</v>
       </c>
       <c r="C12" t="b" s="0">
         <v>1</v>
@@ -632,15 +623,15 @@
         <v>8</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B13" t="s" s="0">
         <v>7</v>
@@ -649,18 +640,18 @@
         <v>1</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B14" t="s" s="0">
         <v>7</v>
@@ -669,258 +660,258 @@
         <v>1</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F14" t="s" s="0">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C15" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D15" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E15" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="F15" t="s" s="0">
         <v>43</v>
-      </c>
-      <c r="E15" t="s" s="0">
-        <v>44</v>
-      </c>
-      <c r="F15" t="s" s="0">
-        <v>45</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C16" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D16" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E16" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="F16" t="s" s="0">
         <v>43</v>
-      </c>
-      <c r="E16" t="s" s="0">
-        <v>48</v>
-      </c>
-      <c r="F16" t="s" s="0">
-        <v>45</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C17" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E17" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F17" t="s" s="0">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C18" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E18" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="F18" t="s" s="0">
         <v>51</v>
-      </c>
-      <c r="B18" t="s" s="0">
-        <v>52</v>
-      </c>
-      <c r="C18" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D18" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="E18" t="s" s="0">
-        <v>29</v>
-      </c>
-      <c r="F18" t="s" s="0">
-        <v>53</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C19" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D19" t="s" s="0">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E19" t="s" s="0">
-        <v>53</v>
+        <v>9</v>
       </c>
       <c r="F19" t="s" s="0">
-        <v>56</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C20" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E20" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="F20" t="s" s="0">
         <v>57</v>
-      </c>
-      <c r="B20" t="s" s="0">
-        <v>58</v>
-      </c>
-      <c r="C20" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D20" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="E20" t="s" s="0">
-        <v>59</v>
-      </c>
-      <c r="F20" t="s" s="0">
-        <v>60</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C21" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D21" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E21" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="F21" t="s" s="0">
         <v>43</v>
-      </c>
-      <c r="E21" t="s" s="0">
-        <v>44</v>
-      </c>
-      <c r="F21" t="s" s="0">
-        <v>45</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C22" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D22" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E22" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="F22" t="s" s="0">
         <v>43</v>
-      </c>
-      <c r="E22" t="s" s="0">
-        <v>61</v>
-      </c>
-      <c r="F22" t="s" s="0">
-        <v>45</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C23" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D23" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E23" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="F23" t="s" s="0">
         <v>43</v>
-      </c>
-      <c r="E23" t="s" s="0">
-        <v>62</v>
-      </c>
-      <c r="F23" t="s" s="0">
-        <v>45</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C24" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D24" t="s" s="0">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="E24" t="s" s="0">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F24" t="s" s="0">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C25" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D25" t="s" s="0">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="E25" t="s" s="0">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F25" t="s" s="0">
-        <v>21</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C26" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D26" t="s" s="0">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="E26" t="s" s="0">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F26" t="s" s="0">
-        <v>53</v>
+        <v>22</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B27" t="s" s="0">
         <v>12</v>
@@ -929,153 +920,153 @@
         <v>1</v>
       </c>
       <c r="D27" t="s" s="0">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="E27" t="s" s="0">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F27" t="s" s="0">
-        <v>26</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
+        <v>66</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>67</v>
+      </c>
+      <c r="C28" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D28" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E28" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="F28" t="s" s="0">
         <v>68</v>
-      </c>
-      <c r="B28" t="s" s="0">
-        <v>69</v>
-      </c>
-      <c r="C28" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D28" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="E28" t="s" s="0">
-        <v>36</v>
-      </c>
-      <c r="F28" t="s" s="0">
-        <v>70</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C29" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="E29" t="s" s="0">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F29" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C30" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D30" t="s" s="0">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="E30" t="s" s="0">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F30" t="s" s="0">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C31" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D31" t="s" s="0">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="E31" t="s" s="0">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F31" t="s" s="0">
-        <v>39</v>
+        <v>18</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="C32" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D32" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E32" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="F32" t="s" s="0">
         <v>73</v>
-      </c>
-      <c r="B32" t="s" s="0">
-        <v>55</v>
-      </c>
-      <c r="C32" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D32" t="s" s="0">
-        <v>40</v>
-      </c>
-      <c r="E32" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="F32" t="s" s="0">
-        <v>29</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C33" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D33" t="s" s="0">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E33" t="s" s="0">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F33" t="s" s="0">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="B34" t="s" s="0">
         <v>76</v>
       </c>
-      <c r="B34" t="s" s="0">
+      <c r="C34" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D34" t="s" s="0">
         <v>77</v>
       </c>
-      <c r="C34" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D34" t="s" s="0">
-        <v>40</v>
-      </c>
       <c r="E34" t="s" s="0">
-        <v>53</v>
+        <v>22</v>
       </c>
       <c r="F34" t="s" s="0">
-        <v>56</v>
+        <v>30</v>
       </c>
     </row>
     <row r="35">
@@ -1083,16 +1074,16 @@
         <v>78</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C35" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D35" t="s" s="0">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="E35" t="s" s="0">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F35" t="s" s="0">
         <v>35</v>
@@ -1109,30 +1100,30 @@
         <v>1</v>
       </c>
       <c r="D36" t="s" s="0">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="E36" t="s" s="0">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F36" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C37" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D37" t="s" s="0">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="E37" t="s" s="0">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="F37" t="s" s="0">
         <v>20</v>
@@ -1140,102 +1131,102 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C38" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D38" t="s" s="0">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E38" t="s" s="0">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="F38" t="s" s="0">
-        <v>17</v>
+        <v>38</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C39" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D39" t="s" s="0">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E39" t="s" s="0">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F39" t="s" s="0">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C40" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D40" t="s" s="0">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E40" t="s" s="0">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F40" t="s" s="0">
-        <v>19</v>
+        <v>27</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C41" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D41" t="s" s="0">
-        <v>75</v>
+        <v>8</v>
       </c>
       <c r="E41" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F41" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C42" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D42" t="s" s="0">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="E42" t="s" s="0">
         <v>10</v>
       </c>
       <c r="F42" t="s" s="0">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="43">
@@ -1243,19 +1234,19 @@
         <v>90</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C43" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D43" t="s" s="0">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="E43" t="s" s="0">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="F43" t="s" s="0">
-        <v>53</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44">
@@ -1263,19 +1254,19 @@
         <v>90</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C44" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D44" t="s" s="0">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="E44" t="s" s="0">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="F44" t="s" s="0">
-        <v>10</v>
+        <v>51</v>
       </c>
     </row>
     <row r="45">
@@ -1283,336 +1274,336 @@
         <v>90</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C45" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D45" t="s" s="0">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E45" t="s" s="0">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F45" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C46" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D46" t="s" s="0">
-        <v>75</v>
+        <v>8</v>
       </c>
       <c r="E46" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F46" t="s" s="0">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C47" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="E47" t="s" s="0">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F47" t="s" s="0">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C48" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D48" t="s" s="0">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="E48" t="s" s="0">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F48" t="s" s="0">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C49" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D49" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E49" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="F49" t="s" s="0">
         <v>43</v>
-      </c>
-      <c r="E49" t="s" s="0">
-        <v>61</v>
-      </c>
-      <c r="F49" t="s" s="0">
-        <v>45</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C50" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D50" t="s" s="0">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="E50" t="s" s="0">
-        <v>95</v>
+        <v>38</v>
       </c>
       <c r="F50" t="s" s="0">
-        <v>96</v>
+        <v>21</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C51" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D51" t="s" s="0">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E51" t="s" s="0">
         <v>21</v>
       </c>
       <c r="F51" t="s" s="0">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C52" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D52" t="s" s="0">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="E52" t="s" s="0">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F52" t="s" s="0">
-        <v>26</v>
+        <v>10</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C53" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D53" t="s" s="0">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="E53" t="s" s="0">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="F53" t="s" s="0">
-        <v>99</v>
+        <v>68</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="0">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C54" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D54" t="s" s="0">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E54" t="s" s="0">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="F54" t="s" s="0">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C55" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D55" t="s" s="0">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="E55" t="s" s="0">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F55" t="s" s="0">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B56" t="s" s="0">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C56" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D56" t="s" s="0">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E56" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F56" t="s" s="0">
-        <v>33</v>
+        <v>73</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="0">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C57" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D57" t="s" s="0">
-        <v>75</v>
+        <v>8</v>
       </c>
       <c r="E57" t="s" s="0">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F57" t="s" s="0">
-        <v>35</v>
+        <v>73</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="0">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B58" t="s" s="0">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C58" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D58" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E58" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="F58" t="s" s="0">
         <v>43</v>
-      </c>
-      <c r="E58" t="s" s="0">
-        <v>44</v>
-      </c>
-      <c r="F58" t="s" s="0">
-        <v>45</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="0">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B59" t="s" s="0">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C59" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D59" t="s" s="0">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="E59" t="s" s="0">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="F59" t="s" s="0">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="0">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B60" t="s" s="0">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C60" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D60" t="s" s="0">
-        <v>107</v>
+        <v>77</v>
       </c>
       <c r="E60" t="s" s="0">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="F60" t="s" s="0">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="0">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B61" t="s" s="0">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C61" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D61" t="s" s="0">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="E61" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F61" t="s" s="0">
         <v>9</v>
@@ -1620,42 +1611,42 @@
     </row>
     <row r="62">
       <c r="A62" t="s" s="0">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B62" t="s" s="0">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C62" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D62" t="s" s="0">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="E62" t="s" s="0">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F62" t="s" s="0">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="0">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B63" t="s" s="0">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C63" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D63" t="s" s="0">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="E63" t="s" s="0">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F63" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: core constraints testing done & fixed minor issues
</commit_message>
<xml_diff>
--- a/java/hello-world/src/main/java/org/acme/schooltimetabling/generated/temp.xlsx
+++ b/java/hello-world/src/main/java/org/acme/schooltimetabling/generated/temp.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="106">
   <si>
     <t>Instructor Name</t>
   </si>
@@ -78,58 +78,61 @@
     <t>MWF 11:00 - 12:00</t>
   </si>
   <si>
+    <t>MWF 15:00 - 16:00</t>
+  </si>
+  <si>
+    <t>MWF 16:00 - 17:00</t>
+  </si>
+  <si>
+    <t>De Moura Canaan, Rodrigo</t>
+  </si>
+  <si>
+    <t>csc480</t>
+  </si>
+  <si>
+    <t>MWF 07:00 - 08:00</t>
+  </si>
+  <si>
+    <t>csc481</t>
+  </si>
+  <si>
+    <t>MWF 12:00 - 13:00</t>
+  </si>
+  <si>
+    <t>Dekhtyar, Alexander M.</t>
+  </si>
+  <si>
+    <t>csc365</t>
+  </si>
+  <si>
+    <t>Eckhardt, Christian</t>
+  </si>
+  <si>
+    <t>csc357</t>
+  </si>
+  <si>
+    <t>csc474</t>
+  </si>
+  <si>
+    <t>TR 12:00 - 13:30</t>
+  </si>
+  <si>
+    <t>TR 13:30 - 15:00</t>
+  </si>
+  <si>
+    <t>Einakian, Sussan</t>
+  </si>
+  <si>
+    <t>csc101</t>
+  </si>
+  <si>
+    <t>MWF 13:00 - 14:00</t>
+  </si>
+  <si>
     <t>MWF 14:00 - 15:00</t>
   </si>
   <si>
-    <t>MWF 15:00 - 16:00</t>
-  </si>
-  <si>
-    <t>De Moura Canaan, Rodrigo</t>
-  </si>
-  <si>
-    <t>csc480</t>
-  </si>
-  <si>
-    <t>MWF 07:00 - 08:00</t>
-  </si>
-  <si>
-    <t>csc481</t>
-  </si>
-  <si>
-    <t>MWF 12:00 - 13:00</t>
-  </si>
-  <si>
-    <t>Dekhtyar, Alexander M.</t>
-  </si>
-  <si>
-    <t>csc365</t>
-  </si>
-  <si>
-    <t>MWF 16:00 - 17:00</t>
-  </si>
-  <si>
-    <t>Eckhardt, Christian</t>
-  </si>
-  <si>
-    <t>csc357</t>
-  </si>
-  <si>
-    <t>csc474</t>
-  </si>
-  <si>
-    <t>TR 12:00 - 13:30</t>
-  </si>
-  <si>
-    <t>TR 13:30 - 15:00</t>
-  </si>
-  <si>
-    <t>Einakian, Sussan</t>
-  </si>
-  <si>
-    <t>csc101</t>
-  </si>
-  <si>
-    <t>MWF 13:00 - 14:00</t>
+    <t>302</t>
   </si>
   <si>
     <t>Frishberg, Daniel</t>
@@ -162,13 +165,16 @@
     <t>csc378</t>
   </si>
   <si>
+    <t>MWF 17:00 - 18:00</t>
+  </si>
+  <si>
     <t>Hristov, Borislav</t>
   </si>
   <si>
     <t>csc448</t>
   </si>
   <si>
-    <t>MWF 17:00 - 18:00</t>
+    <t>MWF 18:00 - 19:00</t>
   </si>
   <si>
     <t>Hsu, Silas</t>
@@ -183,16 +189,16 @@
     <t>csc232</t>
   </si>
   <si>
+    <t>MW 12:00 - 13:00</t>
+  </si>
+  <si>
     <t>MW 13:00 - 14:00</t>
   </si>
   <si>
-    <t>MW 14:00 - 15:00</t>
-  </si>
-  <si>
     <t>MTWR 10:00 - 11:00</t>
   </si>
   <si>
-    <t>MTWR 12:00 - 13:00</t>
+    <t>MTWR 14:00 - 15:00</t>
   </si>
   <si>
     <t>Kalathas, Paris</t>
@@ -207,21 +213,18 @@
     <t>csc477</t>
   </si>
   <si>
+    <t>256</t>
+  </si>
+  <si>
     <t>Keen, Aaron</t>
   </si>
   <si>
-    <t>256</t>
-  </si>
-  <si>
     <t>Khan, Fahim Hasan</t>
   </si>
   <si>
     <t>csc471</t>
   </si>
   <si>
-    <t>MWF 18:00 - 19:00</t>
-  </si>
-  <si>
     <t>Klingenberg, Bernhard J.</t>
   </si>
   <si>
@@ -234,46 +237,40 @@
     <t>csc307</t>
   </si>
   <si>
+    <t>Lindqvist, Ulf Erik</t>
+  </si>
+  <si>
+    <t>csc320</t>
+  </si>
+  <si>
+    <t>192-333</t>
+  </si>
+  <si>
+    <t>Mukherjee, Joydeep</t>
+  </si>
+  <si>
+    <t>csc410</t>
+  </si>
+  <si>
+    <t>257</t>
+  </si>
+  <si>
+    <t>Nico, Phillip L.</t>
+  </si>
+  <si>
+    <t>csc453</t>
+  </si>
+  <si>
     <t>TR 15:00 - 16:30</t>
   </si>
   <si>
-    <t>257</t>
-  </si>
-  <si>
-    <t>Lindqvist, Ulf Erik</t>
-  </si>
-  <si>
-    <t>csc320</t>
-  </si>
-  <si>
-    <t>192-333</t>
-  </si>
-  <si>
-    <t>Mukherjee, Joydeep</t>
-  </si>
-  <si>
-    <t>csc410</t>
-  </si>
-  <si>
-    <t>302</t>
-  </si>
-  <si>
-    <t>Nico, Phillip L.</t>
-  </si>
-  <si>
-    <t>csc453</t>
-  </si>
-  <si>
     <t>Pantoja, Maria</t>
   </si>
   <si>
     <t>csc569</t>
   </si>
   <si>
-    <t>TR 16:00 - 17:30</t>
-  </si>
-  <si>
-    <t>TR 17:30 - 19:00</t>
+    <t>TR 16:30 - 18:00</t>
   </si>
   <si>
     <t>Peterson, Zachary N.J.</t>
@@ -563,18 +560,18 @@
         <v>13</v>
       </c>
       <c r="E9" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="F9" t="s" s="0">
         <v>22</v>
-      </c>
-      <c r="F9" t="s" s="0">
-        <v>30</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="B10" t="s" s="0">
         <v>31</v>
-      </c>
-      <c r="B10" t="s" s="0">
-        <v>32</v>
       </c>
       <c r="C10" t="b" s="0">
         <v>1</v>
@@ -591,10 +588,10 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C11" t="b" s="0">
         <v>1</v>
@@ -603,18 +600,18 @@
         <v>13</v>
       </c>
       <c r="E11" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="F11" t="s" s="0">
         <v>34</v>
-      </c>
-      <c r="F11" t="s" s="0">
-        <v>35</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B12" t="s" s="0">
         <v>36</v>
-      </c>
-      <c r="B12" t="s" s="0">
-        <v>37</v>
       </c>
       <c r="C12" t="b" s="0">
         <v>1</v>
@@ -631,7 +628,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B13" t="s" s="0">
         <v>7</v>
@@ -643,15 +640,15 @@
         <v>8</v>
       </c>
       <c r="E13" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="F13" t="s" s="0">
         <v>38</v>
-      </c>
-      <c r="F13" t="s" s="0">
-        <v>21</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B14" t="s" s="0">
         <v>7</v>
@@ -660,61 +657,61 @@
         <v>1</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="E14" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="F14" t="s" s="0">
         <v>22</v>
-      </c>
-      <c r="F14" t="s" s="0">
-        <v>30</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C15" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E15" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F15" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C16" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F16" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C17" t="b" s="0">
         <v>1</v>
@@ -723,18 +720,18 @@
         <v>13</v>
       </c>
       <c r="E17" t="s" s="0">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F17" t="s" s="0">
-        <v>38</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C18" t="b" s="0">
         <v>1</v>
@@ -743,18 +740,18 @@
         <v>13</v>
       </c>
       <c r="E18" t="s" s="0">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F18" t="s" s="0">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C19" t="b" s="0">
         <v>1</v>
@@ -771,10 +768,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C20" t="b" s="0">
         <v>1</v>
@@ -783,78 +780,78 @@
         <v>13</v>
       </c>
       <c r="E20" t="s" s="0">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F20" t="s" s="0">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C21" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E21" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F21" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C22" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D22" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E22" t="s" s="0">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F22" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C23" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D23" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E23" t="s" s="0">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F23" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C24" t="b" s="0">
         <v>1</v>
@@ -871,10 +868,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C25" t="b" s="0">
         <v>1</v>
@@ -883,35 +880,35 @@
         <v>8</v>
       </c>
       <c r="E25" t="s" s="0">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F25" t="s" s="0">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C26" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D26" t="s" s="0">
-        <v>13</v>
+        <v>66</v>
       </c>
       <c r="E26" t="s" s="0">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F26" t="s" s="0">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B27" t="s" s="0">
         <v>12</v>
@@ -920,7 +917,7 @@
         <v>1</v>
       </c>
       <c r="D27" t="s" s="0">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E27" t="s" s="0">
         <v>9</v>
@@ -931,10 +928,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C28" t="b" s="0">
         <v>1</v>
@@ -943,24 +940,24 @@
         <v>13</v>
       </c>
       <c r="E28" t="s" s="0">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="F28" t="s" s="0">
-        <v>68</v>
+        <v>21</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C29" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E29" t="s" s="0">
         <v>14</v>
@@ -971,36 +968,36 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C30" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D30" t="s" s="0">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E30" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="F30" t="s" s="0">
         <v>34</v>
-      </c>
-      <c r="F30" t="s" s="0">
-        <v>35</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C31" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D31" t="s" s="0">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E31" t="s" s="0">
         <v>10</v>
@@ -1011,10 +1008,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C32" t="b" s="0">
         <v>1</v>
@@ -1023,58 +1020,58 @@
         <v>13</v>
       </c>
       <c r="E32" t="s" s="0">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F32" t="s" s="0">
-        <v>73</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C33" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D33" t="s" s="0">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="E33" t="s" s="0">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F33" t="s" s="0">
-        <v>15</v>
+        <v>27</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="B34" t="s" s="0">
         <v>75</v>
       </c>
-      <c r="B34" t="s" s="0">
+      <c r="C34" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D34" t="s" s="0">
         <v>76</v>
       </c>
-      <c r="C34" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D34" t="s" s="0">
-        <v>77</v>
-      </c>
       <c r="E34" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="F34" t="s" s="0">
         <v>22</v>
-      </c>
-      <c r="F34" t="s" s="0">
-        <v>30</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C35" t="b" s="0">
         <v>1</v>
@@ -1083,24 +1080,24 @@
         <v>8</v>
       </c>
       <c r="E35" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="F35" t="s" s="0">
         <v>34</v>
-      </c>
-      <c r="F35" t="s" s="0">
-        <v>35</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="B36" t="s" s="0">
         <v>78</v>
       </c>
-      <c r="B36" t="s" s="0">
+      <c r="C36" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D36" t="s" s="0">
         <v>79</v>
-      </c>
-      <c r="C36" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D36" t="s" s="0">
-        <v>80</v>
       </c>
       <c r="E36" t="s" s="0">
         <v>14</v>
@@ -1111,42 +1108,42 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="B37" t="s" s="0">
         <v>81</v>
       </c>
-      <c r="B37" t="s" s="0">
+      <c r="C37" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D37" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E37" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="F37" t="s" s="0">
         <v>82</v>
-      </c>
-      <c r="C37" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D37" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="E37" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="F37" t="s" s="0">
-        <v>20</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="B38" t="s" s="0">
         <v>81</v>
       </c>
-      <c r="B38" t="s" s="0">
-        <v>82</v>
-      </c>
       <c r="C38" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D38" t="s" s="0">
-        <v>65</v>
+        <v>39</v>
       </c>
       <c r="E38" t="s" s="0">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F38" t="s" s="0">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="39">
@@ -1163,64 +1160,64 @@
         <v>13</v>
       </c>
       <c r="E39" t="s" s="0">
+        <v>82</v>
+      </c>
+      <c r="F39" t="s" s="0">
         <v>85</v>
-      </c>
-      <c r="F39" t="s" s="0">
-        <v>86</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C40" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D40" t="s" s="0">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E40" t="s" s="0">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F40" t="s" s="0">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="B41" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="B41" t="s" s="0">
-        <v>89</v>
-      </c>
       <c r="C41" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D41" t="s" s="0">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="E41" t="s" s="0">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F41" t="s" s="0">
-        <v>27</v>
+        <v>37</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="B42" t="s" s="0">
         <v>88</v>
       </c>
-      <c r="B42" t="s" s="0">
-        <v>89</v>
-      </c>
       <c r="C42" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D42" t="s" s="0">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E42" t="s" s="0">
         <v>10</v>
@@ -1231,16 +1228,16 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C43" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D43" t="s" s="0">
-        <v>80</v>
+        <v>39</v>
       </c>
       <c r="E43" t="s" s="0">
         <v>9</v>
@@ -1251,36 +1248,36 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C44" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D44" t="s" s="0">
-        <v>80</v>
+        <v>39</v>
       </c>
       <c r="E44" t="s" s="0">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F44" t="s" s="0">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="B45" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="C45" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D45" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="B45" t="s" s="0">
-        <v>61</v>
-      </c>
-      <c r="C45" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D45" t="s" s="0">
-        <v>91</v>
       </c>
       <c r="E45" t="s" s="0">
         <v>14</v>
@@ -1291,10 +1288,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C46" t="b" s="0">
         <v>1</v>
@@ -1303,124 +1300,124 @@
         <v>8</v>
       </c>
       <c r="E46" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="F46" t="s" s="0">
         <v>27</v>
-      </c>
-      <c r="F46" t="s" s="0">
-        <v>38</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C47" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="E47" t="s" s="0">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="F47" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C48" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D48" t="s" s="0">
-        <v>80</v>
+        <v>39</v>
       </c>
       <c r="E48" t="s" s="0">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="F48" t="s" s="0">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="B49" t="s" s="0">
         <v>93</v>
-      </c>
-      <c r="B49" t="s" s="0">
-        <v>94</v>
       </c>
       <c r="C49" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D49" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E49" t="s" s="0">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F49" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C50" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D50" t="s" s="0">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E50" t="s" s="0">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="F50" t="s" s="0">
-        <v>21</v>
+        <v>50</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C51" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D51" t="s" s="0">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E51" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="F51" t="s" s="0">
         <v>21</v>
-      </c>
-      <c r="F51" t="s" s="0">
-        <v>22</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C52" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D52" t="s" s="0">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E52" t="s" s="0">
         <v>9</v>
@@ -1431,10 +1428,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C53" t="b" s="0">
         <v>1</v>
@@ -1443,78 +1440,78 @@
         <v>8</v>
       </c>
       <c r="E53" t="s" s="0">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="F53" t="s" s="0">
-        <v>68</v>
+        <v>37</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="B54" t="s" s="0">
         <v>98</v>
       </c>
-      <c r="B54" t="s" s="0">
-        <v>99</v>
-      </c>
       <c r="C54" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D54" t="s" s="0">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E54" t="s" s="0">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="F54" t="s" s="0">
-        <v>30</v>
+        <v>82</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="B55" t="s" s="0">
         <v>98</v>
       </c>
-      <c r="B55" t="s" s="0">
-        <v>99</v>
-      </c>
       <c r="C55" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D55" t="s" s="0">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E55" t="s" s="0">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F55" t="s" s="0">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B56" t="s" s="0">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C56" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D56" t="s" s="0">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E56" t="s" s="0">
-        <v>35</v>
+        <v>82</v>
       </c>
       <c r="F56" t="s" s="0">
-        <v>73</v>
+        <v>85</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="0">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C57" t="b" s="0">
         <v>1</v>
@@ -1523,44 +1520,44 @@
         <v>8</v>
       </c>
       <c r="E57" t="s" s="0">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F57" t="s" s="0">
-        <v>73</v>
+        <v>82</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="0">
+        <v>100</v>
+      </c>
+      <c r="B58" t="s" s="0">
         <v>101</v>
-      </c>
-      <c r="B58" t="s" s="0">
-        <v>102</v>
       </c>
       <c r="C58" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D58" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E58" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F58" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="0">
+        <v>102</v>
+      </c>
+      <c r="B59" t="s" s="0">
         <v>103</v>
       </c>
-      <c r="B59" t="s" s="0">
-        <v>104</v>
-      </c>
       <c r="C59" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D59" t="s" s="0">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E59" t="s" s="0">
         <v>10</v>
@@ -1571,36 +1568,36 @@
     </row>
     <row r="60">
       <c r="A60" t="s" s="0">
+        <v>102</v>
+      </c>
+      <c r="B60" t="s" s="0">
         <v>103</v>
       </c>
-      <c r="B60" t="s" s="0">
-        <v>104</v>
-      </c>
       <c r="C60" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D60" t="s" s="0">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E60" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="F60" t="s" s="0">
         <v>38</v>
-      </c>
-      <c r="F60" t="s" s="0">
-        <v>21</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="0">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B61" t="s" s="0">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C61" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D61" t="s" s="0">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E61" t="s" s="0">
         <v>25</v>
@@ -1611,42 +1608,42 @@
     </row>
     <row r="62">
       <c r="A62" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="B62" t="s" s="0">
         <v>105</v>
       </c>
-      <c r="B62" t="s" s="0">
-        <v>106</v>
-      </c>
       <c r="C62" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D62" t="s" s="0">
-        <v>65</v>
+        <v>8</v>
       </c>
       <c r="E62" t="s" s="0">
-        <v>30</v>
+        <v>82</v>
       </c>
       <c r="F62" t="s" s="0">
-        <v>51</v>
+        <v>85</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="B63" t="s" s="0">
         <v>105</v>
       </c>
-      <c r="B63" t="s" s="0">
-        <v>106</v>
-      </c>
       <c r="C63" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D63" t="s" s="0">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E63" t="s" s="0">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="F63" t="s" s="0">
-        <v>20</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implemented and tested prime time constraint and added simulate annealing
</commit_message>
<xml_diff>
--- a/java/hello-world/src/main/java/org/acme/schooltimetabling/generated/temp.xlsx
+++ b/java/hello-world/src/main/java/org/acme/schooltimetabling/generated/temp.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="112">
   <si>
     <t>Instructor Name</t>
   </si>
@@ -39,256 +39,274 @@
     <t>csc202</t>
   </si>
   <si>
+    <t>302</t>
+  </si>
+  <si>
+    <t>MWF 09:00 - 10:00</t>
+  </si>
+  <si>
+    <t>MWF 10:00 - 11:00</t>
+  </si>
+  <si>
+    <t>Beard, Stephen Robert</t>
+  </si>
+  <si>
+    <t>csc430</t>
+  </si>
+  <si>
+    <t>257</t>
+  </si>
+  <si>
+    <t>TR 08:00 - 09:30</t>
+  </si>
+  <si>
+    <t>TR 09:30 - 11:00</t>
+  </si>
+  <si>
+    <t>Bellardo, John Michael</t>
+  </si>
+  <si>
+    <t>csc454</t>
+  </si>
+  <si>
+    <t>TR 15:00 - 16:30</t>
+  </si>
+  <si>
+    <t>TR 16:30 - 18:00</t>
+  </si>
+  <si>
+    <t>Clements, John B.</t>
+  </si>
+  <si>
+    <t>232A</t>
+  </si>
+  <si>
+    <t>MWF 15:00 - 16:00</t>
+  </si>
+  <si>
+    <t>MWF 16:00 - 17:00</t>
+  </si>
+  <si>
+    <t>De Moura Canaan, Rodrigo</t>
+  </si>
+  <si>
+    <t>csc480</t>
+  </si>
+  <si>
+    <t>192-206</t>
+  </si>
+  <si>
+    <t>MWF 17:00 - 18:00</t>
+  </si>
+  <si>
+    <t>csc481</t>
+  </si>
+  <si>
+    <t>255</t>
+  </si>
+  <si>
+    <t>Dekhtyar, Alexander M.</t>
+  </si>
+  <si>
+    <t>csc365</t>
+  </si>
+  <si>
     <t>301</t>
   </si>
   <si>
+    <t>Eckhardt, Christian</t>
+  </si>
+  <si>
+    <t>csc357</t>
+  </si>
+  <si>
+    <t>csc474</t>
+  </si>
+  <si>
+    <t>Einakian, Sussan</t>
+  </si>
+  <si>
+    <t>csc101</t>
+  </si>
+  <si>
+    <t>MWF 11:00 - 12:00</t>
+  </si>
+  <si>
     <t>MWF 08:00 - 09:00</t>
   </si>
   <si>
-    <t>MWF 09:00 - 10:00</t>
-  </si>
-  <si>
-    <t>Beard, Stephen Robert</t>
-  </si>
-  <si>
-    <t>csc430</t>
-  </si>
-  <si>
-    <t>255</t>
-  </si>
-  <si>
-    <t>TR 08:00 - 09:30</t>
-  </si>
-  <si>
-    <t>TR 09:30 - 11:00</t>
-  </si>
-  <si>
-    <t>Bellardo, John Michael</t>
-  </si>
-  <si>
-    <t>csc454</t>
-  </si>
-  <si>
-    <t>MWF 10:00 - 11:00</t>
-  </si>
-  <si>
-    <t>Clements, John B.</t>
-  </si>
-  <si>
-    <t>MWF 11:00 - 12:00</t>
-  </si>
-  <si>
-    <t>MWF 15:00 - 16:00</t>
-  </si>
-  <si>
-    <t>MWF 16:00 - 17:00</t>
-  </si>
-  <si>
-    <t>De Moura Canaan, Rodrigo</t>
-  </si>
-  <si>
-    <t>csc480</t>
+    <t>Frishberg, Daniel</t>
+  </si>
+  <si>
+    <t>csc445</t>
+  </si>
+  <si>
+    <t>LECTURE_ONLY</t>
+  </si>
+  <si>
+    <t>MTWR 16:00 - 17:00</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Gonzalez Sanchez, Javier</t>
+  </si>
+  <si>
+    <t>csc570</t>
+  </si>
+  <si>
+    <t>Grow, April Marie</t>
+  </si>
+  <si>
+    <t>csc378</t>
+  </si>
+  <si>
+    <t>MWF 18:00 - 19:00</t>
+  </si>
+  <si>
+    <t>Hristov, Borislav</t>
+  </si>
+  <si>
+    <t>csc448</t>
   </si>
   <si>
     <t>MWF 07:00 - 08:00</t>
   </si>
   <si>
-    <t>csc481</t>
+    <t>Hsu, Silas</t>
+  </si>
+  <si>
+    <t>csc437</t>
+  </si>
+  <si>
+    <t>TR 18:30 - 20:00</t>
+  </si>
+  <si>
+    <t>TR 20:00 - 21:30</t>
+  </si>
+  <si>
+    <t>Jones, Brian Thomas</t>
+  </si>
+  <si>
+    <t>csc232</t>
+  </si>
+  <si>
+    <t>WF 16:00 - 17:00</t>
+  </si>
+  <si>
+    <t>WF 17:00 - 18:00</t>
+  </si>
+  <si>
+    <t>TR 16:00 - 18:00</t>
+  </si>
+  <si>
+    <t>TR 14:00 - 16:00</t>
+  </si>
+  <si>
+    <t>TR 18:00 - 20:00</t>
+  </si>
+  <si>
+    <t>Kalathas, Paris</t>
+  </si>
+  <si>
+    <t>csc203</t>
+  </si>
+  <si>
+    <t>Kazerouni, Ayaan</t>
+  </si>
+  <si>
+    <t>csc477</t>
+  </si>
+  <si>
+    <t>Keen, Aaron</t>
+  </si>
+  <si>
+    <t>Khan, Fahim Hasan</t>
+  </si>
+  <si>
+    <t>csc471</t>
+  </si>
+  <si>
+    <t>TR 17:00 - 18:30</t>
+  </si>
+  <si>
+    <t>Klingenberg, Bernhard J.</t>
+  </si>
+  <si>
+    <t>csc406</t>
+  </si>
+  <si>
+    <t>256</t>
+  </si>
+  <si>
+    <t>Kubiak, Kenneth E.</t>
+  </si>
+  <si>
+    <t>csc307</t>
+  </si>
+  <si>
+    <t>192-333</t>
+  </si>
+  <si>
+    <t>TR 13:30 - 15:00</t>
+  </si>
+  <si>
+    <t>Lindqvist, Ulf Erik</t>
+  </si>
+  <si>
+    <t>csc320</t>
+  </si>
+  <si>
+    <t>Mukherjee, Joydeep</t>
+  </si>
+  <si>
+    <t>csc410</t>
+  </si>
+  <si>
+    <t>TR 12:00 - 13:30</t>
+  </si>
+  <si>
+    <t>Nico, Phillip L.</t>
+  </si>
+  <si>
+    <t>csc453</t>
+  </si>
+  <si>
+    <t>Pantoja, Maria</t>
+  </si>
+  <si>
+    <t>csc569</t>
+  </si>
+  <si>
+    <t>TR 18:00 - 19:30</t>
+  </si>
+  <si>
+    <t>TR 19:30 - 21:00</t>
+  </si>
+  <si>
+    <t>Peterson, Zachary N.J.</t>
   </si>
   <si>
     <t>MWF 12:00 - 13:00</t>
   </si>
   <si>
-    <t>Dekhtyar, Alexander M.</t>
-  </si>
-  <si>
-    <t>csc365</t>
-  </si>
-  <si>
-    <t>Eckhardt, Christian</t>
-  </si>
-  <si>
-    <t>csc357</t>
-  </si>
-  <si>
-    <t>csc474</t>
-  </si>
-  <si>
-    <t>TR 12:00 - 13:30</t>
-  </si>
-  <si>
-    <t>TR 13:30 - 15:00</t>
-  </si>
-  <si>
-    <t>Einakian, Sussan</t>
-  </si>
-  <si>
-    <t>csc101</t>
+    <t>Pierce, Lucas Shane</t>
+  </si>
+  <si>
+    <t>csc466</t>
+  </si>
+  <si>
+    <t>Rathi, Anita</t>
+  </si>
+  <si>
+    <t>Rivera, Vanessa</t>
   </si>
   <si>
     <t>MWF 13:00 - 14:00</t>
   </si>
   <si>
     <t>MWF 14:00 - 15:00</t>
-  </si>
-  <si>
-    <t>302</t>
-  </si>
-  <si>
-    <t>Frishberg, Daniel</t>
-  </si>
-  <si>
-    <t>csc445</t>
-  </si>
-  <si>
-    <t>LECTURE_ONLY</t>
-  </si>
-  <si>
-    <t>MTWR 09:00 - 10:00</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Gonzalez Sanchez, Javier</t>
-  </si>
-  <si>
-    <t>csc570</t>
-  </si>
-  <si>
-    <t>MTWR 11:00 - 12:00</t>
-  </si>
-  <si>
-    <t>Grow, April Marie</t>
-  </si>
-  <si>
-    <t>csc378</t>
-  </si>
-  <si>
-    <t>MWF 17:00 - 18:00</t>
-  </si>
-  <si>
-    <t>Hristov, Borislav</t>
-  </si>
-  <si>
-    <t>csc448</t>
-  </si>
-  <si>
-    <t>MWF 18:00 - 19:00</t>
-  </si>
-  <si>
-    <t>Hsu, Silas</t>
-  </si>
-  <si>
-    <t>csc437</t>
-  </si>
-  <si>
-    <t>Jones, Brian Thomas</t>
-  </si>
-  <si>
-    <t>csc232</t>
-  </si>
-  <si>
-    <t>MW 12:00 - 13:00</t>
-  </si>
-  <si>
-    <t>MW 13:00 - 14:00</t>
-  </si>
-  <si>
-    <t>MTWR 10:00 - 11:00</t>
-  </si>
-  <si>
-    <t>MTWR 14:00 - 15:00</t>
-  </si>
-  <si>
-    <t>Kalathas, Paris</t>
-  </si>
-  <si>
-    <t>csc203</t>
-  </si>
-  <si>
-    <t>Kazerouni, Ayaan</t>
-  </si>
-  <si>
-    <t>csc477</t>
-  </si>
-  <si>
-    <t>256</t>
-  </si>
-  <si>
-    <t>Keen, Aaron</t>
-  </si>
-  <si>
-    <t>Khan, Fahim Hasan</t>
-  </si>
-  <si>
-    <t>csc471</t>
-  </si>
-  <si>
-    <t>Klingenberg, Bernhard J.</t>
-  </si>
-  <si>
-    <t>csc406</t>
-  </si>
-  <si>
-    <t>Kubiak, Kenneth E.</t>
-  </si>
-  <si>
-    <t>csc307</t>
-  </si>
-  <si>
-    <t>Lindqvist, Ulf Erik</t>
-  </si>
-  <si>
-    <t>csc320</t>
-  </si>
-  <si>
-    <t>192-333</t>
-  </si>
-  <si>
-    <t>Mukherjee, Joydeep</t>
-  </si>
-  <si>
-    <t>csc410</t>
-  </si>
-  <si>
-    <t>257</t>
-  </si>
-  <si>
-    <t>Nico, Phillip L.</t>
-  </si>
-  <si>
-    <t>csc453</t>
-  </si>
-  <si>
-    <t>TR 15:00 - 16:30</t>
-  </si>
-  <si>
-    <t>Pantoja, Maria</t>
-  </si>
-  <si>
-    <t>csc569</t>
-  </si>
-  <si>
-    <t>TR 16:30 - 18:00</t>
-  </si>
-  <si>
-    <t>Peterson, Zachary N.J.</t>
-  </si>
-  <si>
-    <t>Pierce, Lucas Shane</t>
-  </si>
-  <si>
-    <t>csc466</t>
-  </si>
-  <si>
-    <t>Rathi, Anita</t>
-  </si>
-  <si>
-    <t>232A</t>
-  </si>
-  <si>
-    <t>Rivera, Vanessa</t>
   </si>
   <si>
     <t>Rwebangira, Mugizi Robert</t>
@@ -460,15 +478,15 @@
         <v>13</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s" s="0">
         <v>12</v>
@@ -477,18 +495,18 @@
         <v>1</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>7</v>
@@ -500,135 +518,135 @@
         <v>8</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="C7" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="E7" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="B7" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="C7" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D7" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="E7" t="s" s="0">
-        <v>25</v>
-      </c>
       <c r="F7" t="s" s="0">
-        <v>9</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C8" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>27</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C9" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C10" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C11" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="F11" t="s" s="0">
-        <v>34</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C12" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="E12" t="s" s="0">
         <v>10</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>18</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B13" t="s" s="0">
         <v>7</v>
@@ -637,18 +655,18 @@
         <v>1</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>38</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B14" t="s" s="0">
         <v>7</v>
@@ -657,13 +675,13 @@
         <v>1</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F14" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15">
@@ -700,7 +718,7 @@
         <v>42</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="F16" t="s" s="0">
         <v>44</v>
@@ -708,87 +726,87 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="B17" t="s" s="0">
         <v>48</v>
       </c>
-      <c r="B17" t="s" s="0">
+      <c r="C17" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E17" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="F17" t="s" s="0">
         <v>49</v>
-      </c>
-      <c r="C17" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D17" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="E17" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="F17" t="s" s="0">
-        <v>50</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="B18" t="s" s="0">
         <v>51</v>
       </c>
-      <c r="B18" t="s" s="0">
+      <c r="C18" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="E18" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="C18" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D18" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="E18" t="s" s="0">
-        <v>50</v>
-      </c>
       <c r="F18" t="s" s="0">
-        <v>53</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="B19" t="s" s="0">
         <v>54</v>
       </c>
-      <c r="B19" t="s" s="0">
+      <c r="C19" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="E19" t="s" s="0">
         <v>55</v>
       </c>
-      <c r="C19" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D19" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="E19" t="s" s="0">
-        <v>9</v>
-      </c>
       <c r="F19" t="s" s="0">
-        <v>10</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C20" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D20" t="s" s="0">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="E20" t="s" s="0">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F20" t="s" s="0">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B21" t="s" s="0">
         <v>41</v>
@@ -800,7 +818,7 @@
         <v>42</v>
       </c>
       <c r="E21" t="s" s="0">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="F21" t="s" s="0">
         <v>44</v>
@@ -808,7 +826,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B22" t="s" s="0">
         <v>41</v>
@@ -820,7 +838,7 @@
         <v>42</v>
       </c>
       <c r="E22" t="s" s="0">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F22" t="s" s="0">
         <v>44</v>
@@ -828,7 +846,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B23" t="s" s="0">
         <v>41</v>
@@ -840,7 +858,7 @@
         <v>42</v>
       </c>
       <c r="E23" t="s" s="0">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F23" t="s" s="0">
         <v>44</v>
@@ -848,67 +866,67 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C24" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D24" t="s" s="0">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="E24" t="s" s="0">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F24" t="s" s="0">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C25" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D25" t="s" s="0">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="E25" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F25" t="s" s="0">
-        <v>50</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C26" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D26" t="s" s="0">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="E26" t="s" s="0">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F26" t="s" s="0">
-        <v>20</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B27" t="s" s="0">
         <v>12</v>
@@ -917,47 +935,47 @@
         <v>1</v>
       </c>
       <c r="D27" t="s" s="0">
-        <v>66</v>
+        <v>29</v>
       </c>
       <c r="E27" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="F27" t="s" s="0">
         <v>9</v>
-      </c>
-      <c r="F27" t="s" s="0">
-        <v>10</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C28" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D28" t="s" s="0">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E28" t="s" s="0">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="F28" t="s" s="0">
-        <v>21</v>
+        <v>55</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C29" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E29" t="s" s="0">
         <v>14</v>
@@ -968,150 +986,150 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C30" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D30" t="s" s="0">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E30" t="s" s="0">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="F30" t="s" s="0">
-        <v>34</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C31" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D31" t="s" s="0">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E31" t="s" s="0">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="F31" t="s" s="0">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C32" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D32" t="s" s="0">
-        <v>13</v>
+        <v>77</v>
       </c>
       <c r="E32" t="s" s="0">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="F32" t="s" s="0">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C33" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D33" t="s" s="0">
-        <v>66</v>
+        <v>13</v>
       </c>
       <c r="E33" t="s" s="0">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="F33" t="s" s="0">
-        <v>27</v>
+        <v>18</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C34" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D34" t="s" s="0">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E34" t="s" s="0">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F34" t="s" s="0">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C35" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D35" t="s" s="0">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="E35" t="s" s="0">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="F35" t="s" s="0">
-        <v>34</v>
+        <v>15</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B36" t="s" s="0">
+        <v>82</v>
+      </c>
+      <c r="C36" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D36" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="E36" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="F36" t="s" s="0">
         <v>78</v>
-      </c>
-      <c r="C36" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D36" t="s" s="0">
-        <v>79</v>
-      </c>
-      <c r="E36" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="F36" t="s" s="0">
-        <v>15</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C37" t="b" s="0">
         <v>1</v>
@@ -1120,164 +1138,164 @@
         <v>13</v>
       </c>
       <c r="E37" t="s" s="0">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F37" t="s" s="0">
-        <v>82</v>
+        <v>9</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C38" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D38" t="s" s="0">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="E38" t="s" s="0">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F38" t="s" s="0">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C39" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D39" t="s" s="0">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="E39" t="s" s="0">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="F39" t="s" s="0">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C40" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D40" t="s" s="0">
-        <v>66</v>
+        <v>21</v>
       </c>
       <c r="E40" t="s" s="0">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="F40" t="s" s="0">
-        <v>22</v>
+        <v>91</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C41" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D41" t="s" s="0">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E41" t="s" s="0">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="F41" t="s" s="0">
-        <v>37</v>
+        <v>91</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C42" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D42" t="s" s="0">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="E42" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="F42" t="s" s="0">
         <v>10</v>
-      </c>
-      <c r="F42" t="s" s="0">
-        <v>18</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C43" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D43" t="s" s="0">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="E43" t="s" s="0">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="F43" t="s" s="0">
-        <v>10</v>
+        <v>27</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C44" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D44" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="E44" t="s" s="0">
         <v>39</v>
       </c>
-      <c r="E44" t="s" s="0">
-        <v>22</v>
-      </c>
       <c r="F44" t="s" s="0">
-        <v>50</v>
+        <v>9</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C45" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D45" t="s" s="0">
-        <v>90</v>
+        <v>8</v>
       </c>
       <c r="E45" t="s" s="0">
         <v>14</v>
@@ -1288,70 +1306,70 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C46" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D46" t="s" s="0">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="E46" t="s" s="0">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="F46" t="s" s="0">
-        <v>27</v>
+        <v>9</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C47" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="E47" t="s" s="0">
-        <v>38</v>
+        <v>96</v>
       </c>
       <c r="F47" t="s" s="0">
-        <v>21</v>
+        <v>97</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C48" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D48" t="s" s="0">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="E48" t="s" s="0">
         <v>10</v>
       </c>
       <c r="F48" t="s" s="0">
-        <v>18</v>
+        <v>38</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="C49" t="b" s="0">
         <v>0</v>
@@ -1360,7 +1378,7 @@
         <v>42</v>
       </c>
       <c r="E49" t="s" s="0">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F49" t="s" s="0">
         <v>44</v>
@@ -1368,70 +1386,70 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C50" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D50" t="s" s="0">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="E50" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F50" t="s" s="0">
-        <v>50</v>
+        <v>27</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C51" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D51" t="s" s="0">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="E51" t="s" s="0">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F51" t="s" s="0">
-        <v>21</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C52" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D52" t="s" s="0">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="E52" t="s" s="0">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F52" t="s" s="0">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C53" t="b" s="0">
         <v>1</v>
@@ -1440,98 +1458,98 @@
         <v>8</v>
       </c>
       <c r="E53" t="s" s="0">
-        <v>27</v>
+        <v>71</v>
       </c>
       <c r="F53" t="s" s="0">
-        <v>37</v>
+        <v>55</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="0">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C54" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D54" t="s" s="0">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="E54" t="s" s="0">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F54" t="s" s="0">
-        <v>82</v>
+        <v>9</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C55" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D55" t="s" s="0">
-        <v>76</v>
+        <v>13</v>
       </c>
       <c r="E55" t="s" s="0">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F55" t="s" s="0">
-        <v>15</v>
+        <v>27</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="B56" t="s" s="0">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C56" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D56" t="s" s="0">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="E56" t="s" s="0">
-        <v>82</v>
+        <v>18</v>
       </c>
       <c r="F56" t="s" s="0">
-        <v>85</v>
+        <v>19</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="0">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C57" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D57" t="s" s="0">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="E57" t="s" s="0">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="F57" t="s" s="0">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="0">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B58" t="s" s="0">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="C58" t="b" s="0">
         <v>0</v>
@@ -1548,39 +1566,39 @@
     </row>
     <row r="59">
       <c r="A59" t="s" s="0">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="B59" t="s" s="0">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C59" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D59" t="s" s="0">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E59" t="s" s="0">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F59" t="s" s="0">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="0">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="B60" t="s" s="0">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C60" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D60" t="s" s="0">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E60" t="s" s="0">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="F60" t="s" s="0">
         <v>38</v>
@@ -1588,62 +1606,62 @@
     </row>
     <row r="61">
       <c r="A61" t="s" s="0">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B61" t="s" s="0">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C61" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D61" t="s" s="0">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E61" t="s" s="0">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F61" t="s" s="0">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s" s="0">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B62" t="s" s="0">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C62" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D62" t="s" s="0">
-        <v>8</v>
+        <v>74</v>
       </c>
       <c r="E62" t="s" s="0">
-        <v>82</v>
+        <v>52</v>
       </c>
       <c r="F62" t="s" s="0">
-        <v>85</v>
+        <v>39</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="0">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B63" t="s" s="0">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C63" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D63" t="s" s="0">
-        <v>79</v>
+        <v>26</v>
       </c>
       <c r="E63" t="s" s="0">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="F63" t="s" s="0">
-        <v>34</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: tested and implemented studio spacing constraint
</commit_message>
<xml_diff>
--- a/java/hello-world/src/main/java/org/acme/schooltimetabling/generated/temp.xlsx
+++ b/java/hello-world/src/main/java/org/acme/schooltimetabling/generated/temp.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="117">
   <si>
     <t>Instructor Name</t>
   </si>
@@ -39,234 +39,255 @@
     <t>csc202</t>
   </si>
   <si>
+    <t>301</t>
+  </si>
+  <si>
+    <t>MWF 10:00 - 11:00</t>
+  </si>
+  <si>
+    <t>MWF 11:00 - 12:00</t>
+  </si>
+  <si>
+    <t>Beard, Stephen Robert</t>
+  </si>
+  <si>
+    <t>csc430</t>
+  </si>
+  <si>
+    <t>192-206</t>
+  </si>
+  <si>
+    <t>TR 08:00 - 09:30</t>
+  </si>
+  <si>
+    <t>TR 09:30 - 11:00</t>
+  </si>
+  <si>
+    <t>Bellardo, John Michael</t>
+  </si>
+  <si>
+    <t>csc454</t>
+  </si>
+  <si>
     <t>302</t>
   </si>
   <si>
+    <t>TR 15:00 - 16:30</t>
+  </si>
+  <si>
+    <t>TR 16:30 - 18:00</t>
+  </si>
+  <si>
+    <t>Clements, John B.</t>
+  </si>
+  <si>
+    <t>232A</t>
+  </si>
+  <si>
+    <t>MWF 15:00 - 16:00</t>
+  </si>
+  <si>
+    <t>MWF 16:00 - 17:00</t>
+  </si>
+  <si>
+    <t>De Moura Canaan, Rodrigo</t>
+  </si>
+  <si>
+    <t>csc480</t>
+  </si>
+  <si>
+    <t>255</t>
+  </si>
+  <si>
+    <t>MWF 07:00 - 08:00</t>
+  </si>
+  <si>
+    <t>MWF 08:00 - 09:00</t>
+  </si>
+  <si>
+    <t>csc481</t>
+  </si>
+  <si>
+    <t>TR 16:00 - 17:30</t>
+  </si>
+  <si>
+    <t>TR 17:30 - 19:00</t>
+  </si>
+  <si>
+    <t>Dekhtyar, Alexander M.</t>
+  </si>
+  <si>
+    <t>csc365</t>
+  </si>
+  <si>
+    <t>Eckhardt, Christian</t>
+  </si>
+  <si>
+    <t>csc357</t>
+  </si>
+  <si>
+    <t>csc474</t>
+  </si>
+  <si>
+    <t>Einakian, Sussan</t>
+  </si>
+  <si>
+    <t>csc101</t>
+  </si>
+  <si>
+    <t>MWF 13:00 - 14:00</t>
+  </si>
+  <si>
+    <t>MWF 14:00 - 15:00</t>
+  </si>
+  <si>
     <t>MWF 09:00 - 10:00</t>
   </si>
   <si>
-    <t>MWF 10:00 - 11:00</t>
-  </si>
-  <si>
-    <t>Beard, Stephen Robert</t>
-  </si>
-  <si>
-    <t>csc430</t>
+    <t>Frishberg, Daniel</t>
+  </si>
+  <si>
+    <t>csc445</t>
+  </si>
+  <si>
+    <t>LECTURE_ONLY</t>
+  </si>
+  <si>
+    <t>MTWR 16:00 - 17:00</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Gonzalez Sanchez, Javier</t>
+  </si>
+  <si>
+    <t>csc570</t>
+  </si>
+  <si>
+    <t>MTWR 15:00 - 16:00</t>
+  </si>
+  <si>
+    <t>Grow, April Marie</t>
+  </si>
+  <si>
+    <t>csc378</t>
+  </si>
+  <si>
+    <t>TR 18:00 - 19:30</t>
+  </si>
+  <si>
+    <t>Hristov, Borislav</t>
+  </si>
+  <si>
+    <t>csc448</t>
+  </si>
+  <si>
+    <t>TR 18:30 - 20:00</t>
+  </si>
+  <si>
+    <t>TR 20:00 - 21:30</t>
+  </si>
+  <si>
+    <t>Hsu, Silas</t>
+  </si>
+  <si>
+    <t>csc437</t>
+  </si>
+  <si>
+    <t>256</t>
+  </si>
+  <si>
+    <t>TR 19:00 - 20:30</t>
+  </si>
+  <si>
+    <t>Jones, Brian Thomas</t>
+  </si>
+  <si>
+    <t>csc232</t>
+  </si>
+  <si>
+    <t>192-333</t>
+  </si>
+  <si>
+    <t>WF 17:00 - 18:00</t>
+  </si>
+  <si>
+    <t>WF 18:00 - 19:00</t>
+  </si>
+  <si>
+    <t>TR 16:00 - 18:00</t>
+  </si>
+  <si>
+    <t>TR 18:00 - 20:00</t>
+  </si>
+  <si>
+    <t>TR 14:00 - 16:00</t>
+  </si>
+  <si>
+    <t>Kalathas, Paris</t>
+  </si>
+  <si>
+    <t>csc203</t>
+  </si>
+  <si>
+    <t>Kazerouni, Ayaan</t>
+  </si>
+  <si>
+    <t>MWF 17:00 - 18:00</t>
+  </si>
+  <si>
+    <t>csc477</t>
+  </si>
+  <si>
+    <t>Keen, Aaron</t>
+  </si>
+  <si>
+    <t>Khan, Fahim Hasan</t>
+  </si>
+  <si>
+    <t>csc471</t>
+  </si>
+  <si>
+    <t>MWF 18:00 - 19:00</t>
+  </si>
+  <si>
+    <t>MWF 19:00 - 20:00</t>
+  </si>
+  <si>
+    <t>Klingenberg, Bernhard J.</t>
+  </si>
+  <si>
+    <t>csc406</t>
+  </si>
+  <si>
+    <t>Kubiak, Kenneth E.</t>
+  </si>
+  <si>
+    <t>csc307</t>
+  </si>
+  <si>
+    <t>TR 13:30 - 15:00</t>
+  </si>
+  <si>
+    <t>Lindqvist, Ulf Erik</t>
+  </si>
+  <si>
+    <t>csc320</t>
+  </si>
+  <si>
+    <t>Mukherjee, Joydeep</t>
+  </si>
+  <si>
+    <t>TR 12:00 - 13:30</t>
+  </si>
+  <si>
+    <t>csc410</t>
   </si>
   <si>
     <t>257</t>
   </si>
   <si>
-    <t>TR 08:00 - 09:30</t>
-  </si>
-  <si>
-    <t>TR 09:30 - 11:00</t>
-  </si>
-  <si>
-    <t>Bellardo, John Michael</t>
-  </si>
-  <si>
-    <t>csc454</t>
-  </si>
-  <si>
-    <t>TR 15:00 - 16:30</t>
-  </si>
-  <si>
-    <t>TR 16:30 - 18:00</t>
-  </si>
-  <si>
-    <t>Clements, John B.</t>
-  </si>
-  <si>
-    <t>232A</t>
-  </si>
-  <si>
-    <t>MWF 15:00 - 16:00</t>
-  </si>
-  <si>
-    <t>MWF 16:00 - 17:00</t>
-  </si>
-  <si>
-    <t>De Moura Canaan, Rodrigo</t>
-  </si>
-  <si>
-    <t>csc480</t>
-  </si>
-  <si>
-    <t>192-206</t>
-  </si>
-  <si>
-    <t>MWF 17:00 - 18:00</t>
-  </si>
-  <si>
-    <t>csc481</t>
-  </si>
-  <si>
-    <t>255</t>
-  </si>
-  <si>
-    <t>Dekhtyar, Alexander M.</t>
-  </si>
-  <si>
-    <t>csc365</t>
-  </si>
-  <si>
-    <t>301</t>
-  </si>
-  <si>
-    <t>Eckhardt, Christian</t>
-  </si>
-  <si>
-    <t>csc357</t>
-  </si>
-  <si>
-    <t>csc474</t>
-  </si>
-  <si>
-    <t>Einakian, Sussan</t>
-  </si>
-  <si>
-    <t>csc101</t>
-  </si>
-  <si>
-    <t>MWF 11:00 - 12:00</t>
-  </si>
-  <si>
-    <t>MWF 08:00 - 09:00</t>
-  </si>
-  <si>
-    <t>Frishberg, Daniel</t>
-  </si>
-  <si>
-    <t>csc445</t>
-  </si>
-  <si>
-    <t>LECTURE_ONLY</t>
-  </si>
-  <si>
-    <t>MTWR 16:00 - 17:00</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Gonzalez Sanchez, Javier</t>
-  </si>
-  <si>
-    <t>csc570</t>
-  </si>
-  <si>
-    <t>Grow, April Marie</t>
-  </si>
-  <si>
-    <t>csc378</t>
-  </si>
-  <si>
-    <t>MWF 18:00 - 19:00</t>
-  </si>
-  <si>
-    <t>Hristov, Borislav</t>
-  </si>
-  <si>
-    <t>csc448</t>
-  </si>
-  <si>
-    <t>MWF 07:00 - 08:00</t>
-  </si>
-  <si>
-    <t>Hsu, Silas</t>
-  </si>
-  <si>
-    <t>csc437</t>
-  </si>
-  <si>
-    <t>TR 18:30 - 20:00</t>
-  </si>
-  <si>
-    <t>TR 20:00 - 21:30</t>
-  </si>
-  <si>
-    <t>Jones, Brian Thomas</t>
-  </si>
-  <si>
-    <t>csc232</t>
-  </si>
-  <si>
-    <t>WF 16:00 - 17:00</t>
-  </si>
-  <si>
-    <t>WF 17:00 - 18:00</t>
-  </si>
-  <si>
-    <t>TR 16:00 - 18:00</t>
-  </si>
-  <si>
-    <t>TR 14:00 - 16:00</t>
-  </si>
-  <si>
-    <t>TR 18:00 - 20:00</t>
-  </si>
-  <si>
-    <t>Kalathas, Paris</t>
-  </si>
-  <si>
-    <t>csc203</t>
-  </si>
-  <si>
-    <t>Kazerouni, Ayaan</t>
-  </si>
-  <si>
-    <t>csc477</t>
-  </si>
-  <si>
-    <t>Keen, Aaron</t>
-  </si>
-  <si>
-    <t>Khan, Fahim Hasan</t>
-  </si>
-  <si>
-    <t>csc471</t>
-  </si>
-  <si>
-    <t>TR 17:00 - 18:30</t>
-  </si>
-  <si>
-    <t>Klingenberg, Bernhard J.</t>
-  </si>
-  <si>
-    <t>csc406</t>
-  </si>
-  <si>
-    <t>256</t>
-  </si>
-  <si>
-    <t>Kubiak, Kenneth E.</t>
-  </si>
-  <si>
-    <t>csc307</t>
-  </si>
-  <si>
-    <t>192-333</t>
-  </si>
-  <si>
-    <t>TR 13:30 - 15:00</t>
-  </si>
-  <si>
-    <t>Lindqvist, Ulf Erik</t>
-  </si>
-  <si>
-    <t>csc320</t>
-  </si>
-  <si>
-    <t>Mukherjee, Joydeep</t>
-  </si>
-  <si>
-    <t>csc410</t>
-  </si>
-  <si>
-    <t>TR 12:00 - 13:30</t>
-  </si>
-  <si>
     <t>Nico, Phillip L.</t>
   </si>
   <si>
@@ -279,40 +300,34 @@
     <t>csc569</t>
   </si>
   <si>
-    <t>TR 18:00 - 19:30</t>
+    <t>Peterson, Zachary N.J.</t>
+  </si>
+  <si>
+    <t>Pierce, Lucas Shane</t>
+  </si>
+  <si>
+    <t>csc466</t>
+  </si>
+  <si>
+    <t>MWF 12:00 - 13:00</t>
+  </si>
+  <si>
+    <t>Rathi, Anita</t>
+  </si>
+  <si>
+    <t>Rivera, Vanessa</t>
   </si>
   <si>
     <t>TR 19:30 - 21:00</t>
   </si>
   <si>
-    <t>Peterson, Zachary N.J.</t>
-  </si>
-  <si>
-    <t>MWF 12:00 - 13:00</t>
-  </si>
-  <si>
-    <t>Pierce, Lucas Shane</t>
-  </si>
-  <si>
-    <t>csc466</t>
-  </si>
-  <si>
-    <t>Rathi, Anita</t>
-  </si>
-  <si>
-    <t>Rivera, Vanessa</t>
-  </si>
-  <si>
-    <t>MWF 13:00 - 14:00</t>
-  </si>
-  <si>
-    <t>MWF 14:00 - 15:00</t>
-  </si>
-  <si>
     <t>Rwebangira, Mugizi Robert</t>
   </si>
   <si>
     <t>csc566</t>
+  </si>
+  <si>
+    <t>TR 17:00 - 19:00</t>
   </si>
   <si>
     <t>csc349</t>
@@ -475,18 +490,18 @@
         <v>1</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s" s="0">
         <v>12</v>
@@ -495,18 +510,18 @@
         <v>1</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>10</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>7</v>
@@ -515,107 +530,107 @@
         <v>1</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C7" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C8" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>19</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C9" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C10" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C11" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E11" t="s" s="0">
         <v>14</v>
@@ -626,27 +641,27 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C12" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B13" t="s" s="0">
         <v>7</v>
@@ -655,18 +670,18 @@
         <v>1</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>9</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B14" t="s" s="0">
         <v>7</v>
@@ -675,258 +690,258 @@
         <v>1</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F14" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C15" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E15" t="s" s="0">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F15" t="s" s="0">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C16" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="F16" t="s" s="0">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C17" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E17" t="s" s="0">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F17" t="s" s="0">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C18" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D18" t="s" s="0">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="E18" t="s" s="0">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F18" t="s" s="0">
-        <v>39</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C19" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D19" t="s" s="0">
-        <v>26</v>
+        <v>60</v>
       </c>
       <c r="E19" t="s" s="0">
-        <v>55</v>
+        <v>32</v>
       </c>
       <c r="F19" t="s" s="0">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C20" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D20" t="s" s="0">
-        <v>29</v>
+        <v>64</v>
       </c>
       <c r="E20" t="s" s="0">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F20" t="s" s="0">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C21" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E21" t="s" s="0">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="F21" t="s" s="0">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C22" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D22" t="s" s="0">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E22" t="s" s="0">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="F22" t="s" s="0">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C23" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D23" t="s" s="0">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E23" t="s" s="0">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F23" t="s" s="0">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="C24" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D24" t="s" s="0">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E24" t="s" s="0">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F24" t="s" s="0">
-        <v>15</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="C25" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D25" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E25" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F25" t="s" s="0">
-        <v>27</v>
+        <v>73</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C26" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D26" t="s" s="0">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E26" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="F26" t="s" s="0">
         <v>10</v>
-      </c>
-      <c r="F26" t="s" s="0">
-        <v>38</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="B27" t="s" s="0">
         <v>12</v>
@@ -935,367 +950,367 @@
         <v>1</v>
       </c>
       <c r="D27" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E27" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="E27" t="s" s="0">
-        <v>39</v>
-      </c>
       <c r="F27" t="s" s="0">
-        <v>9</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="C28" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D28" t="s" s="0">
-        <v>21</v>
+        <v>60</v>
       </c>
       <c r="E28" t="s" s="0">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="F28" t="s" s="0">
-        <v>55</v>
+        <v>79</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="C29" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="E29" t="s" s="0">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F29" t="s" s="0">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="C30" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D30" t="s" s="0">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="E30" t="s" s="0">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F30" t="s" s="0">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="C31" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D31" t="s" s="0">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="E31" t="s" s="0">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="F31" t="s" s="0">
-        <v>9</v>
+        <v>24</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C32" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D32" t="s" s="0">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="E32" t="s" s="0">
-        <v>14</v>
+        <v>84</v>
       </c>
       <c r="F32" t="s" s="0">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C33" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D33" t="s" s="0">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E33" t="s" s="0">
-        <v>78</v>
+        <v>14</v>
       </c>
       <c r="F33" t="s" s="0">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C34" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D34" t="s" s="0">
-        <v>77</v>
+        <v>13</v>
       </c>
       <c r="E34" t="s" s="0">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F34" t="s" s="0">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C35" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D35" t="s" s="0">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E35" t="s" s="0">
-        <v>14</v>
+        <v>88</v>
       </c>
       <c r="F35" t="s" s="0">
-        <v>15</v>
+        <v>84</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C36" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D36" t="s" s="0">
-        <v>26</v>
+        <v>90</v>
       </c>
       <c r="E36" t="s" s="0">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="F36" t="s" s="0">
-        <v>78</v>
+        <v>15</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="C37" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D37" t="s" s="0">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="E37" t="s" s="0">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="F37" t="s" s="0">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="C38" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D38" t="s" s="0">
-        <v>13</v>
+        <v>90</v>
       </c>
       <c r="E38" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F38" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="C39" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D39" t="s" s="0">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="E39" t="s" s="0">
-        <v>88</v>
+        <v>20</v>
       </c>
       <c r="F39" t="s" s="0">
-        <v>89</v>
+        <v>53</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="C40" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D40" t="s" s="0">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E40" t="s" s="0">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="F40" t="s" s="0">
-        <v>91</v>
+        <v>24</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C41" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D41" t="s" s="0">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="E41" t="s" s="0">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="F41" t="s" s="0">
-        <v>91</v>
+        <v>40</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C42" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D42" t="s" s="0">
-        <v>29</v>
+        <v>64</v>
       </c>
       <c r="E42" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="F42" t="s" s="0">
         <v>9</v>
-      </c>
-      <c r="F42" t="s" s="0">
-        <v>10</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C43" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D43" t="s" s="0">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="E43" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F43" t="s" s="0">
-        <v>27</v>
+        <v>73</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C44" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D44" t="s" s="0">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="E44" t="s" s="0">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="F44" t="s" s="0">
-        <v>9</v>
+        <v>42</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="C45" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D45" t="s" s="0">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="E45" t="s" s="0">
         <v>14</v>
@@ -1306,50 +1321,50 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C46" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D46" t="s" s="0">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E46" t="s" s="0">
-        <v>39</v>
+        <v>84</v>
       </c>
       <c r="F46" t="s" s="0">
-        <v>9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C47" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E47" t="s" s="0">
-        <v>96</v>
+        <v>53</v>
       </c>
       <c r="F47" t="s" s="0">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C48" t="b" s="0">
         <v>1</v>
@@ -1358,310 +1373,310 @@
         <v>8</v>
       </c>
       <c r="E48" t="s" s="0">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F48" t="s" s="0">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C49" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D49" t="s" s="0">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E49" t="s" s="0">
-        <v>61</v>
+        <v>104</v>
       </c>
       <c r="F49" t="s" s="0">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="C50" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D50" t="s" s="0">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="E50" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F50" t="s" s="0">
-        <v>27</v>
+        <v>73</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="C51" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D51" t="s" s="0">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E51" t="s" s="0">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="F51" t="s" s="0">
-        <v>9</v>
+        <v>24</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="C52" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D52" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="E52" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="E52" t="s" s="0">
-        <v>22</v>
-      </c>
       <c r="F52" t="s" s="0">
-        <v>23</v>
+        <v>42</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C53" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D53" t="s" s="0">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="E53" t="s" s="0">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="F53" t="s" s="0">
-        <v>55</v>
+        <v>79</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="0">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C54" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D54" t="s" s="0">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="E54" t="s" s="0">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="F54" t="s" s="0">
-        <v>9</v>
+        <v>73</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C55" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D55" t="s" s="0">
-        <v>13</v>
+        <v>90</v>
       </c>
       <c r="E55" t="s" s="0">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F55" t="s" s="0">
-        <v>27</v>
+        <v>42</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
+        <v>110</v>
+      </c>
+      <c r="B56" t="s" s="0">
         <v>105</v>
       </c>
-      <c r="B56" t="s" s="0">
-        <v>100</v>
-      </c>
       <c r="C56" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D56" t="s" s="0">
-        <v>26</v>
+        <v>90</v>
       </c>
       <c r="E56" t="s" s="0">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F56" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="0">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C57" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D57" t="s" s="0">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="E57" t="s" s="0">
-        <v>83</v>
+        <v>42</v>
       </c>
       <c r="F57" t="s" s="0">
-        <v>78</v>
+        <v>9</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="0">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B58" t="s" s="0">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="C58" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D58" t="s" s="0">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E58" t="s" s="0">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F58" t="s" s="0">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="0">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B59" t="s" s="0">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="C59" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D59" t="s" s="0">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="E59" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F59" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="0">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B60" t="s" s="0">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="C60" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D60" t="s" s="0">
-        <v>77</v>
+        <v>13</v>
       </c>
       <c r="E60" t="s" s="0">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="F60" t="s" s="0">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="0">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B61" t="s" s="0">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="C61" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D61" t="s" s="0">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="E61" t="s" s="0">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="F61" t="s" s="0">
-        <v>10</v>
+        <v>29</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s" s="0">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B62" t="s" s="0">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="C62" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D62" t="s" s="0">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="E62" t="s" s="0">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="F62" t="s" s="0">
-        <v>39</v>
+        <v>73</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="0">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B63" t="s" s="0">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="C63" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D63" t="s" s="0">
-        <v>26</v>
+        <v>64</v>
       </c>
       <c r="E63" t="s" s="0">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="F63" t="s" s="0">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: code clean up, bug fixes, and more documentation
</commit_message>
<xml_diff>
--- a/java/hello-world/src/main/java/org/acme/schooltimetabling/generated/temp.xlsx
+++ b/java/hello-world/src/main/java/org/acme/schooltimetabling/generated/temp.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="114">
   <si>
     <t>Instructor Name</t>
   </si>
@@ -39,73 +39,205 @@
     <t>csc202</t>
   </si>
   <si>
+    <t>302</t>
+  </si>
+  <si>
+    <t>MWF 09:00 - 10:00</t>
+  </si>
+  <si>
+    <t>MWF 10:00 - 11:00</t>
+  </si>
+  <si>
+    <t>Beard, Stephen Robert</t>
+  </si>
+  <si>
+    <t>csc430</t>
+  </si>
+  <si>
+    <t>TR 08:00 - 09:30</t>
+  </si>
+  <si>
+    <t>TR 09:30 - 11:00</t>
+  </si>
+  <si>
+    <t>Bellardo, John Michael</t>
+  </si>
+  <si>
+    <t>csc454</t>
+  </si>
+  <si>
+    <t>192-333</t>
+  </si>
+  <si>
+    <t>TR 15:00 - 16:30</t>
+  </si>
+  <si>
+    <t>TR 16:30 - 18:00</t>
+  </si>
+  <si>
+    <t>Clements, John B.</t>
+  </si>
+  <si>
+    <t>MWF 11:00 - 12:00</t>
+  </si>
+  <si>
+    <t>MWF 12:00 - 13:00</t>
+  </si>
+  <si>
+    <t>TR 13:30 - 15:00</t>
+  </si>
+  <si>
+    <t>De Moura Canaan, Rodrigo</t>
+  </si>
+  <si>
+    <t>csc480</t>
+  </si>
+  <si>
     <t>301</t>
   </si>
   <si>
-    <t>MWF 10:00 - 11:00</t>
-  </si>
-  <si>
-    <t>MWF 11:00 - 12:00</t>
-  </si>
-  <si>
-    <t>Beard, Stephen Robert</t>
-  </si>
-  <si>
-    <t>csc430</t>
+    <t>MWF 07:00 - 08:00</t>
+  </si>
+  <si>
+    <t>MWF 08:00 - 09:00</t>
+  </si>
+  <si>
+    <t>csc481</t>
+  </si>
+  <si>
+    <t>255</t>
+  </si>
+  <si>
+    <t>MWF 16:00 - 17:00</t>
+  </si>
+  <si>
+    <t>MWF 17:00 - 18:00</t>
+  </si>
+  <si>
+    <t>Dekhtyar, Alexander M.</t>
+  </si>
+  <si>
+    <t>csc365</t>
+  </si>
+  <si>
+    <t>MWF 15:00 - 16:00</t>
+  </si>
+  <si>
+    <t>Eckhardt, Christian</t>
+  </si>
+  <si>
+    <t>csc357</t>
+  </si>
+  <si>
+    <t>csc474</t>
+  </si>
+  <si>
+    <t>Einakian, Sussan</t>
+  </si>
+  <si>
+    <t>csc101</t>
+  </si>
+  <si>
+    <t>MWF 13:00 - 14:00</t>
+  </si>
+  <si>
+    <t>MWF 14:00 - 15:00</t>
+  </si>
+  <si>
+    <t>232A</t>
+  </si>
+  <si>
+    <t>Frishberg, Daniel</t>
+  </si>
+  <si>
+    <t>csc445</t>
+  </si>
+  <si>
+    <t>LECTURE_ONLY</t>
+  </si>
+  <si>
+    <t>MTWR 15:00 - 16:00</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Gonzalez Sanchez, Javier</t>
+  </si>
+  <si>
+    <t>csc570</t>
+  </si>
+  <si>
+    <t>Grow, April Marie</t>
+  </si>
+  <si>
+    <t>csc378</t>
+  </si>
+  <si>
+    <t>MWF 18:00 - 19:00</t>
+  </si>
+  <si>
+    <t>MWF 19:00 - 20:00</t>
+  </si>
+  <si>
+    <t>Hristov, Borislav</t>
+  </si>
+  <si>
+    <t>csc448</t>
+  </si>
+  <si>
+    <t>Hsu, Silas</t>
+  </si>
+  <si>
+    <t>csc437</t>
+  </si>
+  <si>
+    <t>257</t>
+  </si>
+  <si>
+    <t>Jones, Brian Thomas</t>
+  </si>
+  <si>
+    <t>csc232</t>
   </si>
   <si>
     <t>192-206</t>
   </si>
   <si>
-    <t>TR 08:00 - 09:30</t>
-  </si>
-  <si>
-    <t>TR 09:30 - 11:00</t>
-  </si>
-  <si>
-    <t>Bellardo, John Michael</t>
-  </si>
-  <si>
-    <t>csc454</t>
-  </si>
-  <si>
-    <t>302</t>
-  </si>
-  <si>
-    <t>TR 15:00 - 16:30</t>
-  </si>
-  <si>
-    <t>TR 16:30 - 18:00</t>
-  </si>
-  <si>
-    <t>Clements, John B.</t>
-  </si>
-  <si>
-    <t>232A</t>
-  </si>
-  <si>
-    <t>MWF 15:00 - 16:00</t>
-  </si>
-  <si>
-    <t>MWF 16:00 - 17:00</t>
-  </si>
-  <si>
-    <t>De Moura Canaan, Rodrigo</t>
-  </si>
-  <si>
-    <t>csc480</t>
-  </si>
-  <si>
-    <t>255</t>
-  </si>
-  <si>
-    <t>MWF 07:00 - 08:00</t>
-  </si>
-  <si>
-    <t>MWF 08:00 - 09:00</t>
-  </si>
-  <si>
-    <t>csc481</t>
+    <t>WF 15:00 - 16:00</t>
+  </si>
+  <si>
+    <t>WF 16:00 - 17:00</t>
+  </si>
+  <si>
+    <t>MTWR 19:00 - 20:00</t>
+  </si>
+  <si>
+    <t>MTWR 17:00 - 18:00</t>
+  </si>
+  <si>
+    <t>MTWR 18:00 - 19:00</t>
+  </si>
+  <si>
+    <t>Kalathas, Paris</t>
+  </si>
+  <si>
+    <t>csc203</t>
+  </si>
+  <si>
+    <t>Kazerouni, Ayaan</t>
+  </si>
+  <si>
+    <t>csc477</t>
+  </si>
+  <si>
+    <t>Keen, Aaron</t>
+  </si>
+  <si>
+    <t>Khan, Fahim Hasan</t>
+  </si>
+  <si>
+    <t>csc471</t>
   </si>
   <si>
     <t>TR 16:00 - 17:30</t>
@@ -114,244 +246,103 @@
     <t>TR 17:30 - 19:00</t>
   </si>
   <si>
-    <t>Dekhtyar, Alexander M.</t>
-  </si>
-  <si>
-    <t>csc365</t>
-  </si>
-  <si>
-    <t>Eckhardt, Christian</t>
-  </si>
-  <si>
-    <t>csc357</t>
-  </si>
-  <si>
-    <t>csc474</t>
-  </si>
-  <si>
-    <t>Einakian, Sussan</t>
-  </si>
-  <si>
-    <t>csc101</t>
-  </si>
-  <si>
-    <t>MWF 13:00 - 14:00</t>
-  </si>
-  <si>
-    <t>MWF 14:00 - 15:00</t>
-  </si>
-  <si>
-    <t>MWF 09:00 - 10:00</t>
-  </si>
-  <si>
-    <t>Frishberg, Daniel</t>
-  </si>
-  <si>
-    <t>csc445</t>
-  </si>
-  <si>
-    <t>LECTURE_ONLY</t>
+    <t>Klingenberg, Bernhard J.</t>
+  </si>
+  <si>
+    <t>csc406</t>
+  </si>
+  <si>
+    <t>256</t>
+  </si>
+  <si>
+    <t>TR 12:00 - 13:30</t>
+  </si>
+  <si>
+    <t>Kubiak, Kenneth E.</t>
+  </si>
+  <si>
+    <t>csc307</t>
+  </si>
+  <si>
+    <t>Lindqvist, Ulf Erik</t>
+  </si>
+  <si>
+    <t>csc320</t>
+  </si>
+  <si>
+    <t>Mukherjee, Joydeep</t>
+  </si>
+  <si>
+    <t>csc410</t>
+  </si>
+  <si>
+    <t>Nico, Phillip L.</t>
+  </si>
+  <si>
+    <t>csc453</t>
+  </si>
+  <si>
+    <t>Pantoja, Maria</t>
+  </si>
+  <si>
+    <t>csc569</t>
+  </si>
+  <si>
+    <t>TR 18:00 - 19:30</t>
+  </si>
+  <si>
+    <t>TR 19:30 - 21:00</t>
+  </si>
+  <si>
+    <t>Peterson, Zachary N.J.</t>
+  </si>
+  <si>
+    <t>Pierce, Lucas Shane</t>
+  </si>
+  <si>
+    <t>csc466</t>
+  </si>
+  <si>
+    <t>Rathi, Anita</t>
+  </si>
+  <si>
+    <t>Rivera, Vanessa</t>
+  </si>
+  <si>
+    <t>Rwebangira, Mugizi Robert</t>
+  </si>
+  <si>
+    <t>csc566</t>
+  </si>
+  <si>
+    <t>TR 17:00 - 19:00</t>
+  </si>
+  <si>
+    <t>csc349</t>
+  </si>
+  <si>
+    <t>Schmitt, Paul</t>
+  </si>
+  <si>
+    <t>Siu, Christopher E.</t>
+  </si>
+  <si>
+    <t>Stanchev, Lubomir Petrov</t>
+  </si>
+  <si>
+    <t>csc366</t>
+  </si>
+  <si>
+    <t>Teo, Ka Yaw</t>
+  </si>
+  <si>
+    <t>Ventura, Jonathan Daniel</t>
+  </si>
+  <si>
+    <t>csc587</t>
   </si>
   <si>
     <t>MTWR 16:00 - 17:00</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Gonzalez Sanchez, Javier</t>
-  </si>
-  <si>
-    <t>csc570</t>
-  </si>
-  <si>
-    <t>MTWR 15:00 - 16:00</t>
-  </si>
-  <si>
-    <t>Grow, April Marie</t>
-  </si>
-  <si>
-    <t>csc378</t>
-  </si>
-  <si>
-    <t>TR 18:00 - 19:30</t>
-  </si>
-  <si>
-    <t>Hristov, Borislav</t>
-  </si>
-  <si>
-    <t>csc448</t>
-  </si>
-  <si>
-    <t>TR 18:30 - 20:00</t>
-  </si>
-  <si>
-    <t>TR 20:00 - 21:30</t>
-  </si>
-  <si>
-    <t>Hsu, Silas</t>
-  </si>
-  <si>
-    <t>csc437</t>
-  </si>
-  <si>
-    <t>256</t>
-  </si>
-  <si>
-    <t>TR 19:00 - 20:30</t>
-  </si>
-  <si>
-    <t>Jones, Brian Thomas</t>
-  </si>
-  <si>
-    <t>csc232</t>
-  </si>
-  <si>
-    <t>192-333</t>
-  </si>
-  <si>
-    <t>WF 17:00 - 18:00</t>
-  </si>
-  <si>
-    <t>WF 18:00 - 19:00</t>
-  </si>
-  <si>
-    <t>TR 16:00 - 18:00</t>
-  </si>
-  <si>
-    <t>TR 18:00 - 20:00</t>
-  </si>
-  <si>
-    <t>TR 14:00 - 16:00</t>
-  </si>
-  <si>
-    <t>Kalathas, Paris</t>
-  </si>
-  <si>
-    <t>csc203</t>
-  </si>
-  <si>
-    <t>Kazerouni, Ayaan</t>
-  </si>
-  <si>
-    <t>MWF 17:00 - 18:00</t>
-  </si>
-  <si>
-    <t>csc477</t>
-  </si>
-  <si>
-    <t>Keen, Aaron</t>
-  </si>
-  <si>
-    <t>Khan, Fahim Hasan</t>
-  </si>
-  <si>
-    <t>csc471</t>
-  </si>
-  <si>
-    <t>MWF 18:00 - 19:00</t>
-  </si>
-  <si>
-    <t>MWF 19:00 - 20:00</t>
-  </si>
-  <si>
-    <t>Klingenberg, Bernhard J.</t>
-  </si>
-  <si>
-    <t>csc406</t>
-  </si>
-  <si>
-    <t>Kubiak, Kenneth E.</t>
-  </si>
-  <si>
-    <t>csc307</t>
-  </si>
-  <si>
-    <t>TR 13:30 - 15:00</t>
-  </si>
-  <si>
-    <t>Lindqvist, Ulf Erik</t>
-  </si>
-  <si>
-    <t>csc320</t>
-  </si>
-  <si>
-    <t>Mukherjee, Joydeep</t>
-  </si>
-  <si>
-    <t>TR 12:00 - 13:30</t>
-  </si>
-  <si>
-    <t>csc410</t>
-  </si>
-  <si>
-    <t>257</t>
-  </si>
-  <si>
-    <t>Nico, Phillip L.</t>
-  </si>
-  <si>
-    <t>csc453</t>
-  </si>
-  <si>
-    <t>Pantoja, Maria</t>
-  </si>
-  <si>
-    <t>csc569</t>
-  </si>
-  <si>
-    <t>Peterson, Zachary N.J.</t>
-  </si>
-  <si>
-    <t>Pierce, Lucas Shane</t>
-  </si>
-  <si>
-    <t>csc466</t>
-  </si>
-  <si>
-    <t>MWF 12:00 - 13:00</t>
-  </si>
-  <si>
-    <t>Rathi, Anita</t>
-  </si>
-  <si>
-    <t>Rivera, Vanessa</t>
-  </si>
-  <si>
-    <t>TR 19:30 - 21:00</t>
-  </si>
-  <si>
-    <t>Rwebangira, Mugizi Robert</t>
-  </si>
-  <si>
-    <t>csc566</t>
-  </si>
-  <si>
-    <t>TR 17:00 - 19:00</t>
-  </si>
-  <si>
-    <t>csc349</t>
-  </si>
-  <si>
-    <t>Schmitt, Paul</t>
-  </si>
-  <si>
-    <t>Siu, Christopher E.</t>
-  </si>
-  <si>
-    <t>Stanchev, Lubomir Petrov</t>
-  </si>
-  <si>
-    <t>csc366</t>
-  </si>
-  <si>
-    <t>Teo, Ka Yaw</t>
-  </si>
-  <si>
-    <t>Ventura, Jonathan Daniel</t>
-  </si>
-  <si>
-    <t>csc587</t>
   </si>
   <si>
     <t>Yocam, Eric Wayne</t>
@@ -470,38 +461,38 @@
         <v>1</v>
       </c>
       <c r="D3" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="E3" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="E3" t="s" s="0">
+      <c r="F3" t="s" s="0">
         <v>14</v>
-      </c>
-      <c r="F3" t="s" s="0">
-        <v>15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="C4" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s" s="0">
         <v>17</v>
       </c>
-      <c r="C4" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D4" t="s" s="0">
+      <c r="E4" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="E4" t="s" s="0">
+      <c r="F4" t="s" s="0">
         <v>19</v>
-      </c>
-      <c r="F4" t="s" s="0">
-        <v>20</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s" s="0">
         <v>12</v>
@@ -510,18 +501,18 @@
         <v>1</v>
       </c>
       <c r="D5" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s" s="0">
         <v>22</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="F5" t="s" s="0">
-        <v>24</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>7</v>
@@ -530,47 +521,47 @@
         <v>1</v>
       </c>
       <c r="D6" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="F6" t="s" s="0">
         <v>18</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="F6" t="s" s="0">
-        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="C7" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="C7" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D7" t="s" s="0">
+      <c r="E7" t="s" s="0">
         <v>27</v>
       </c>
-      <c r="E7" t="s" s="0">
+      <c r="F7" t="s" s="0">
         <v>28</v>
-      </c>
-      <c r="F7" t="s" s="0">
-        <v>29</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B8" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="C8" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s" s="0">
         <v>30</v>
-      </c>
-      <c r="C8" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D8" t="s" s="0">
-        <v>22</v>
       </c>
       <c r="E8" t="s" s="0">
         <v>31</v>
@@ -590,21 +581,21 @@
         <v>1</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>24</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C10" t="b" s="0">
         <v>1</v>
@@ -613,55 +604,55 @@
         <v>8</v>
       </c>
       <c r="E10" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="F10" t="s" s="0">
         <v>19</v>
-      </c>
-      <c r="F10" t="s" s="0">
-        <v>20</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C11" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E11" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F11" t="s" s="0">
         <v>14</v>
-      </c>
-      <c r="F11" t="s" s="0">
-        <v>15</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C12" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B13" t="s" s="0">
         <v>7</v>
@@ -670,18 +661,18 @@
         <v>1</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>42</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B14" t="s" s="0">
         <v>7</v>
@@ -690,53 +681,53 @@
         <v>1</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="F14" t="s" s="0">
-        <v>24</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C15" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E15" t="s" s="0">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F15" t="s" s="0">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C16" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F16" t="s" s="0">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17">
@@ -750,198 +741,198 @@
         <v>1</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E17" t="s" s="0">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="F17" t="s" s="0">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C18" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D18" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="E18" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="E18" t="s" s="0">
-        <v>56</v>
-      </c>
       <c r="F18" t="s" s="0">
-        <v>57</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="B19" t="s" s="0">
         <v>58</v>
       </c>
-      <c r="B19" t="s" s="0">
+      <c r="C19" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D19" t="s" s="0">
         <v>59</v>
-      </c>
-      <c r="C19" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D19" t="s" s="0">
-        <v>60</v>
       </c>
       <c r="E19" t="s" s="0">
         <v>32</v>
       </c>
       <c r="F19" t="s" s="0">
-        <v>61</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="C20" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D20" t="s" s="0">
         <v>62</v>
       </c>
-      <c r="B20" t="s" s="0">
+      <c r="E20" t="s" s="0">
         <v>63</v>
       </c>
-      <c r="C20" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D20" t="s" s="0">
+      <c r="F20" t="s" s="0">
         <v>64</v>
-      </c>
-      <c r="E20" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="F20" t="s" s="0">
-        <v>66</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C21" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E21" t="s" s="0">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F21" t="s" s="0">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C22" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D22" t="s" s="0">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E22" t="s" s="0">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F22" t="s" s="0">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C23" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D23" t="s" s="0">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E23" t="s" s="0">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F23" t="s" s="0">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C24" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D24" t="s" s="0">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E24" t="s" s="0">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F24" t="s" s="0">
-        <v>42</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C25" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D25" t="s" s="0">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E25" t="s" s="0">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F25" t="s" s="0">
-        <v>73</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C26" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D26" t="s" s="0">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="E26" t="s" s="0">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F26" t="s" s="0">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B27" t="s" s="0">
         <v>12</v>
@@ -950,733 +941,733 @@
         <v>1</v>
       </c>
       <c r="D27" t="s" s="0">
-        <v>64</v>
+        <v>26</v>
       </c>
       <c r="E27" t="s" s="0">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F27" t="s" s="0">
-        <v>42</v>
+        <v>21</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
+        <v>73</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C28" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D28" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="E28" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="F28" t="s" s="0">
         <v>76</v>
-      </c>
-      <c r="B28" t="s" s="0">
-        <v>77</v>
-      </c>
-      <c r="C28" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D28" t="s" s="0">
-        <v>60</v>
-      </c>
-      <c r="E28" t="s" s="0">
-        <v>78</v>
-      </c>
-      <c r="F28" t="s" s="0">
-        <v>79</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C29" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="E29" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="F29" t="s" s="0">
         <v>19</v>
-      </c>
-      <c r="F29" t="s" s="0">
-        <v>20</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="B30" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="C30" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D30" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E30" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="B30" t="s" s="0">
-        <v>81</v>
-      </c>
-      <c r="C30" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D30" t="s" s="0">
-        <v>60</v>
-      </c>
-      <c r="E30" t="s" s="0">
-        <v>14</v>
-      </c>
       <c r="F30" t="s" s="0">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="B31" t="s" s="0">
         <v>82</v>
       </c>
-      <c r="B31" t="s" s="0">
-        <v>83</v>
-      </c>
       <c r="C31" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D31" t="s" s="0">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="E31" t="s" s="0">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F31" t="s" s="0">
-        <v>24</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C32" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D32" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E32" t="s" s="0">
-        <v>84</v>
+        <v>10</v>
       </c>
       <c r="F32" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B33" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="C33" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D33" t="s" s="0">
         <v>59</v>
       </c>
-      <c r="C33" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D33" t="s" s="0">
-        <v>22</v>
-      </c>
       <c r="E33" t="s" s="0">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="F33" t="s" s="0">
-        <v>15</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C34" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D34" t="s" s="0">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E34" t="s" s="0">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F34" t="s" s="0">
-        <v>20</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C35" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D35" t="s" s="0">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E35" t="s" s="0">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="F35" t="s" s="0">
-        <v>84</v>
+        <v>23</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C36" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D36" t="s" s="0">
-        <v>90</v>
+        <v>26</v>
       </c>
       <c r="E36" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F36" t="s" s="0">
         <v>14</v>
-      </c>
-      <c r="F36" t="s" s="0">
-        <v>15</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C37" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D37" t="s" s="0">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="E37" t="s" s="0">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="F37" t="s" s="0">
-        <v>10</v>
+        <v>31</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C38" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D38" t="s" s="0">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="E38" t="s" s="0">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F38" t="s" s="0">
-        <v>24</v>
+        <v>9</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C39" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D39" t="s" s="0">
-        <v>13</v>
+        <v>62</v>
       </c>
       <c r="E39" t="s" s="0">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="F39" t="s" s="0">
-        <v>53</v>
+        <v>92</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C40" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D40" t="s" s="0">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="E40" t="s" s="0">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F40" t="s" s="0">
-        <v>24</v>
+        <v>9</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C41" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D41" t="s" s="0">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E41" t="s" s="0">
-        <v>98</v>
+        <v>9</v>
       </c>
       <c r="F41" t="s" s="0">
-        <v>40</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C42" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D42" t="s" s="0">
-        <v>64</v>
+        <v>26</v>
       </c>
       <c r="E42" t="s" s="0">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="F42" t="s" s="0">
-        <v>9</v>
+        <v>22</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C43" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D43" t="s" s="0">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E43" t="s" s="0">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F43" t="s" s="0">
-        <v>73</v>
+        <v>9</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C44" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D44" t="s" s="0">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E44" t="s" s="0">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F44" t="s" s="0">
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C45" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D45" t="s" s="0">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="E45" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F45" t="s" s="0">
         <v>14</v>
-      </c>
-      <c r="F45" t="s" s="0">
-        <v>15</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C46" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D46" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="E46" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="E46" t="s" s="0">
-        <v>84</v>
-      </c>
       <c r="F46" t="s" s="0">
-        <v>19</v>
+        <v>41</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C47" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="E47" t="s" s="0">
-        <v>53</v>
+        <v>28</v>
       </c>
       <c r="F47" t="s" s="0">
-        <v>101</v>
+        <v>9</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C48" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D48" t="s" s="0">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E48" t="s" s="0">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="F48" t="s" s="0">
-        <v>15</v>
+        <v>31</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C49" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D49" t="s" s="0">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E49" t="s" s="0">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F49" t="s" s="0">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C50" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D50" t="s" s="0">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="E50" t="s" s="0">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="F50" t="s" s="0">
-        <v>73</v>
+        <v>53</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C51" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D51" t="s" s="0">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="E51" t="s" s="0">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="F51" t="s" s="0">
-        <v>24</v>
+        <v>31</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C52" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D52" t="s" s="0">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="E52" t="s" s="0">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F52" t="s" s="0">
-        <v>42</v>
+        <v>9</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C53" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D53" t="s" s="0">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E53" t="s" s="0">
-        <v>78</v>
+        <v>53</v>
       </c>
       <c r="F53" t="s" s="0">
-        <v>79</v>
+        <v>54</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="0">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C54" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D54" t="s" s="0">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E54" t="s" s="0">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F54" t="s" s="0">
-        <v>73</v>
+        <v>32</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C55" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D55" t="s" s="0">
-        <v>90</v>
+        <v>59</v>
       </c>
       <c r="E55" t="s" s="0">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F55" t="s" s="0">
-        <v>42</v>
+        <v>9</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B56" t="s" s="0">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C56" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D56" t="s" s="0">
-        <v>90</v>
+        <v>43</v>
       </c>
       <c r="E56" t="s" s="0">
-        <v>19</v>
+        <v>75</v>
       </c>
       <c r="F56" t="s" s="0">
-        <v>20</v>
+        <v>76</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="0">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C57" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D57" t="s" s="0">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="E57" t="s" s="0">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="F57" t="s" s="0">
-        <v>9</v>
+        <v>22</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="0">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B58" t="s" s="0">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C58" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D58" t="s" s="0">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E58" t="s" s="0">
-        <v>46</v>
+        <v>109</v>
       </c>
       <c r="F58" t="s" s="0">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="0">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B59" t="s" s="0">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C59" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D59" t="s" s="0">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E59" t="s" s="0">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="F59" t="s" s="0">
-        <v>24</v>
+        <v>42</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="0">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B60" t="s" s="0">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C60" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D60" t="s" s="0">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E60" t="s" s="0">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F60" t="s" s="0">
-        <v>41</v>
+        <v>31</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="0">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B61" t="s" s="0">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C61" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D61" t="s" s="0">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="E61" t="s" s="0">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="F61" t="s" s="0">
-        <v>29</v>
+        <v>21</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s" s="0">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B62" t="s" s="0">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C62" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D62" t="s" s="0">
-        <v>27</v>
+        <v>79</v>
       </c>
       <c r="E62" t="s" s="0">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F62" t="s" s="0">
-        <v>73</v>
+        <v>32</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="0">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B63" t="s" s="0">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C63" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D63" t="s" s="0">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="E63" t="s" s="0">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="F63" t="s" s="0">
-        <v>10</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: teachers with no survey are scheduled and refactored to include more constants
</commit_message>
<xml_diff>
--- a/java/hello-world/src/main/java/org/acme/schooltimetabling/generated/temp.xlsx
+++ b/java/hello-world/src/main/java/org/acme/schooltimetabling/generated/temp.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="133">
   <si>
     <t>Instructor Name</t>
   </si>
@@ -39,270 +39,303 @@
     <t>csc202</t>
   </si>
   <si>
+    <t>301</t>
+  </si>
+  <si>
+    <t>MWF 08:00 - 09:00</t>
+  </si>
+  <si>
+    <t>MWF 09:00 - 10:00</t>
+  </si>
+  <si>
+    <t>Beard, Stephen Robert</t>
+  </si>
+  <si>
+    <t>csc430</t>
+  </si>
+  <si>
+    <t>192-333</t>
+  </si>
+  <si>
+    <t>TR 08:00 - 09:30</t>
+  </si>
+  <si>
+    <t>TR 09:30 - 11:00</t>
+  </si>
+  <si>
+    <t>Bellardo, John Michael</t>
+  </si>
+  <si>
+    <t>csc454</t>
+  </si>
+  <si>
+    <t>192-206</t>
+  </si>
+  <si>
+    <t>TR 15:00 - 16:30</t>
+  </si>
+  <si>
+    <t>TR 16:30 - 18:00</t>
+  </si>
+  <si>
+    <t>Clements, John B.</t>
+  </si>
+  <si>
+    <t>232A</t>
+  </si>
+  <si>
+    <t>MWF 15:00 - 16:00</t>
+  </si>
+  <si>
+    <t>MWF 16:00 - 17:00</t>
+  </si>
+  <si>
+    <t>TR 12:00 - 13:30</t>
+  </si>
+  <si>
+    <t>TR 13:30 - 15:00</t>
+  </si>
+  <si>
+    <t>De Moura Canaan, Rodrigo</t>
+  </si>
+  <si>
+    <t>csc480</t>
+  </si>
+  <si>
+    <t>255</t>
+  </si>
+  <si>
+    <t>csc481</t>
+  </si>
+  <si>
+    <t>256</t>
+  </si>
+  <si>
+    <t>MWF 18:00 - 19:00</t>
+  </si>
+  <si>
+    <t>MWF 19:00 - 20:00</t>
+  </si>
+  <si>
+    <t>Dekhtyar, Alexander M.</t>
+  </si>
+  <si>
+    <t>csc365</t>
+  </si>
+  <si>
+    <t>257</t>
+  </si>
+  <si>
+    <t>Duran, Kirk Alberto</t>
+  </si>
+  <si>
+    <t>csc101</t>
+  </si>
+  <si>
     <t>302</t>
   </si>
   <si>
-    <t>MWF 09:00 - 10:00</t>
+    <t>MWF 20:00 - 21:00</t>
+  </si>
+  <si>
+    <t>MWF 17:00 - 18:00</t>
+  </si>
+  <si>
+    <t>TR 19:00 - 20:30</t>
+  </si>
+  <si>
+    <t>TR 20:30 - 22:00</t>
+  </si>
+  <si>
+    <t>Eckhardt, Christian</t>
+  </si>
+  <si>
+    <t>csc357</t>
+  </si>
+  <si>
+    <t>csc474</t>
+  </si>
+  <si>
+    <t>Einakian, Sussan</t>
   </si>
   <si>
     <t>MWF 10:00 - 11:00</t>
   </si>
   <si>
-    <t>Beard, Stephen Robert</t>
-  </si>
-  <si>
-    <t>csc430</t>
-  </si>
-  <si>
-    <t>TR 08:00 - 09:30</t>
-  </si>
-  <si>
-    <t>TR 09:30 - 11:00</t>
-  </si>
-  <si>
-    <t>Bellardo, John Michael</t>
-  </si>
-  <si>
-    <t>csc454</t>
-  </si>
-  <si>
-    <t>192-333</t>
-  </si>
-  <si>
-    <t>TR 15:00 - 16:30</t>
-  </si>
-  <si>
-    <t>TR 16:30 - 18:00</t>
-  </si>
-  <si>
-    <t>Clements, John B.</t>
-  </si>
-  <si>
     <t>MWF 11:00 - 12:00</t>
   </si>
   <si>
+    <t>Fang, Dongfeng</t>
+  </si>
+  <si>
+    <t>csc321</t>
+  </si>
+  <si>
+    <t>TR 16:00 - 17:30</t>
+  </si>
+  <si>
+    <t>TR 17:30 - 19:00</t>
+  </si>
+  <si>
+    <t>Frishberg, Daniel</t>
+  </si>
+  <si>
+    <t>csc445</t>
+  </si>
+  <si>
+    <t>LECTURE_ONLY</t>
+  </si>
+  <si>
+    <t>MTWR 15:00 - 16:00</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Gonzalez Sanchez, Javier</t>
+  </si>
+  <si>
+    <t>csc570</t>
+  </si>
+  <si>
+    <t>Grow, April Marie</t>
+  </si>
+  <si>
+    <t>csc378</t>
+  </si>
+  <si>
+    <t>Han, Wei-jer</t>
+  </si>
+  <si>
+    <t>csc225</t>
+  </si>
+  <si>
+    <t>Hartman, Bret Andrew</t>
+  </si>
+  <si>
+    <t>csc422</t>
+  </si>
+  <si>
+    <t>Hristov, Borislav</t>
+  </si>
+  <si>
+    <t>csc448</t>
+  </si>
+  <si>
+    <t>TR 18:00 - 19:30</t>
+  </si>
+  <si>
+    <t>Hsu, Silas</t>
+  </si>
+  <si>
+    <t>csc437</t>
+  </si>
+  <si>
+    <t>Jones, Brian Thomas</t>
+  </si>
+  <si>
+    <t>csc232</t>
+  </si>
+  <si>
+    <t>MW 09:00 - 10:00</t>
+  </si>
+  <si>
+    <t>MW 10:00 - 11:00</t>
+  </si>
+  <si>
+    <t>MTWR 18:00 - 19:00</t>
+  </si>
+  <si>
+    <t>MTWR 17:00 - 18:00</t>
+  </si>
+  <si>
+    <t>MTWR 16:00 - 17:00</t>
+  </si>
+  <si>
+    <t>Kalathas, Paris</t>
+  </si>
+  <si>
+    <t>csc203</t>
+  </si>
+  <si>
+    <t>MWF 14:00 - 15:00</t>
+  </si>
+  <si>
+    <t>Kazerouni, Ayaan</t>
+  </si>
+  <si>
+    <t>csc477</t>
+  </si>
+  <si>
+    <t>Keen, Aaron</t>
+  </si>
+  <si>
+    <t>Khan, Fahim Hasan</t>
+  </si>
+  <si>
+    <t>csc471</t>
+  </si>
+  <si>
+    <t>Klingenberg, Bernhard J.</t>
+  </si>
+  <si>
+    <t>csc406</t>
+  </si>
+  <si>
+    <t>Kubiak, Kenneth E.</t>
+  </si>
+  <si>
+    <t>csc307</t>
+  </si>
+  <si>
+    <t>MWF 13:00 - 14:00</t>
+  </si>
+  <si>
+    <t>Lindqvist, Ulf Erik</t>
+  </si>
+  <si>
+    <t>csc320</t>
+  </si>
+  <si>
+    <t>Mukherjee, Joydeep</t>
+  </si>
+  <si>
+    <t>csc410</t>
+  </si>
+  <si>
+    <t>Nico, Phillip L.</t>
+  </si>
+  <si>
+    <t>csc453</t>
+  </si>
+  <si>
+    <t>Pantoja, Maria</t>
+  </si>
+  <si>
+    <t>csc569</t>
+  </si>
+  <si>
+    <t>TR 19:30 - 21:00</t>
+  </si>
+  <si>
+    <t>Peterson, Zachary N.J.</t>
+  </si>
+  <si>
+    <t>Pierce, Lucas Shane</t>
+  </si>
+  <si>
+    <t>csc466</t>
+  </si>
+  <si>
     <t>MWF 12:00 - 13:00</t>
   </si>
   <si>
-    <t>TR 13:30 - 15:00</t>
-  </si>
-  <si>
-    <t>De Moura Canaan, Rodrigo</t>
-  </si>
-  <si>
-    <t>csc480</t>
-  </si>
-  <si>
-    <t>301</t>
+    <t>Planck, John R.</t>
   </si>
   <si>
     <t>MWF 07:00 - 08:00</t>
   </si>
   <si>
-    <t>MWF 08:00 - 09:00</t>
-  </si>
-  <si>
-    <t>csc481</t>
-  </si>
-  <si>
-    <t>255</t>
-  </si>
-  <si>
-    <t>MWF 16:00 - 17:00</t>
-  </si>
-  <si>
-    <t>MWF 17:00 - 18:00</t>
-  </si>
-  <si>
-    <t>Dekhtyar, Alexander M.</t>
-  </si>
-  <si>
-    <t>csc365</t>
-  </si>
-  <si>
-    <t>MWF 15:00 - 16:00</t>
-  </si>
-  <si>
-    <t>Eckhardt, Christian</t>
-  </si>
-  <si>
-    <t>csc357</t>
-  </si>
-  <si>
-    <t>csc474</t>
-  </si>
-  <si>
-    <t>Einakian, Sussan</t>
-  </si>
-  <si>
-    <t>csc101</t>
-  </si>
-  <si>
-    <t>MWF 13:00 - 14:00</t>
-  </si>
-  <si>
-    <t>MWF 14:00 - 15:00</t>
-  </si>
-  <si>
-    <t>232A</t>
-  </si>
-  <si>
-    <t>Frishberg, Daniel</t>
-  </si>
-  <si>
-    <t>csc445</t>
-  </si>
-  <si>
-    <t>LECTURE_ONLY</t>
-  </si>
-  <si>
-    <t>MTWR 15:00 - 16:00</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Gonzalez Sanchez, Javier</t>
-  </si>
-  <si>
-    <t>csc570</t>
-  </si>
-  <si>
-    <t>Grow, April Marie</t>
-  </si>
-  <si>
-    <t>csc378</t>
-  </si>
-  <si>
-    <t>MWF 18:00 - 19:00</t>
-  </si>
-  <si>
-    <t>MWF 19:00 - 20:00</t>
-  </si>
-  <si>
-    <t>Hristov, Borislav</t>
-  </si>
-  <si>
-    <t>csc448</t>
-  </si>
-  <si>
-    <t>Hsu, Silas</t>
-  </si>
-  <si>
-    <t>csc437</t>
-  </si>
-  <si>
-    <t>257</t>
-  </si>
-  <si>
-    <t>Jones, Brian Thomas</t>
-  </si>
-  <si>
-    <t>csc232</t>
-  </si>
-  <si>
-    <t>192-206</t>
-  </si>
-  <si>
-    <t>WF 15:00 - 16:00</t>
-  </si>
-  <si>
-    <t>WF 16:00 - 17:00</t>
-  </si>
-  <si>
-    <t>MTWR 19:00 - 20:00</t>
-  </si>
-  <si>
-    <t>MTWR 17:00 - 18:00</t>
-  </si>
-  <si>
-    <t>MTWR 18:00 - 19:00</t>
-  </si>
-  <si>
-    <t>Kalathas, Paris</t>
-  </si>
-  <si>
-    <t>csc203</t>
-  </si>
-  <si>
-    <t>Kazerouni, Ayaan</t>
-  </si>
-  <si>
-    <t>csc477</t>
-  </si>
-  <si>
-    <t>Keen, Aaron</t>
-  </si>
-  <si>
-    <t>Khan, Fahim Hasan</t>
-  </si>
-  <si>
-    <t>csc471</t>
-  </si>
-  <si>
-    <t>TR 16:00 - 17:30</t>
-  </si>
-  <si>
-    <t>TR 17:30 - 19:00</t>
-  </si>
-  <si>
-    <t>Klingenberg, Bernhard J.</t>
-  </si>
-  <si>
-    <t>csc406</t>
-  </si>
-  <si>
-    <t>256</t>
-  </si>
-  <si>
-    <t>TR 12:00 - 13:30</t>
-  </si>
-  <si>
-    <t>Kubiak, Kenneth E.</t>
-  </si>
-  <si>
-    <t>csc307</t>
-  </si>
-  <si>
-    <t>Lindqvist, Ulf Erik</t>
-  </si>
-  <si>
-    <t>csc320</t>
-  </si>
-  <si>
-    <t>Mukherjee, Joydeep</t>
-  </si>
-  <si>
-    <t>csc410</t>
-  </si>
-  <si>
-    <t>Nico, Phillip L.</t>
-  </si>
-  <si>
-    <t>csc453</t>
-  </si>
-  <si>
-    <t>Pantoja, Maria</t>
-  </si>
-  <si>
-    <t>csc569</t>
-  </si>
-  <si>
-    <t>TR 18:00 - 19:30</t>
-  </si>
-  <si>
-    <t>TR 19:30 - 21:00</t>
-  </si>
-  <si>
-    <t>Peterson, Zachary N.J.</t>
-  </si>
-  <si>
-    <t>Pierce, Lucas Shane</t>
-  </si>
-  <si>
-    <t>csc466</t>
-  </si>
-  <si>
     <t>Rathi, Anita</t>
   </si>
   <si>
@@ -315,15 +348,27 @@
     <t>csc566</t>
   </si>
   <si>
-    <t>TR 17:00 - 19:00</t>
-  </si>
-  <si>
     <t>csc349</t>
   </si>
   <si>
     <t>Schmitt, Paul</t>
   </si>
   <si>
+    <t>Sisodia, Devkishen</t>
+  </si>
+  <si>
+    <t>csc564</t>
+  </si>
+  <si>
+    <t>csc364</t>
+  </si>
+  <si>
+    <t>TR 17:00 - 18:30</t>
+  </si>
+  <si>
+    <t>TR 18:30 - 20:00</t>
+  </si>
+  <si>
     <t>Siu, Christopher E.</t>
   </si>
   <si>
@@ -336,25 +381,37 @@
     <t>Teo, Ka Yaw</t>
   </si>
   <si>
+    <t>Vargas, Luis E.</t>
+  </si>
+  <si>
     <t>Ventura, Jonathan Daniel</t>
   </si>
   <si>
     <t>csc587</t>
   </si>
   <si>
-    <t>MTWR 16:00 - 17:00</t>
+    <t>Wagner, Michael</t>
+  </si>
+  <si>
+    <t>Wang, Jenny Zheng</t>
+  </si>
+  <si>
+    <t>csc484</t>
   </si>
   <si>
     <t>Yocam, Eric Wayne</t>
   </si>
   <si>
-    <t>csc321</t>
-  </si>
-  <si>
     <t>Zielke, Christopher Patrick</t>
   </si>
   <si>
     <t>csc308</t>
+  </si>
+  <si>
+    <t>laila-abdelhafeez</t>
+  </si>
+  <si>
+    <t>TR 20:00 - 21:30</t>
   </si>
 </sst>
 </file>
@@ -399,7 +456,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F82"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="35.15625" customWidth="true"/>
@@ -461,38 +518,38 @@
         <v>1</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s" s="0">
         <v>12</v>
@@ -501,18 +558,18 @@
         <v>1</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>7</v>
@@ -524,95 +581,95 @@
         <v>8</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C7" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>28</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C8" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C9" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>31</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C10" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>19</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s" s="0">
         <v>38</v>
@@ -621,170 +678,170 @@
         <v>1</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F11" t="s" s="0">
-        <v>14</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="C12" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="C13" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C14" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="F14" t="s" s="0">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C15" t="b" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="E15" t="s" s="0">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F15" t="s" s="0">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>50</v>
+        <v>7</v>
       </c>
       <c r="C16" t="b" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>47</v>
+        <v>9</v>
       </c>
       <c r="F16" t="s" s="0">
-        <v>48</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>52</v>
+        <v>7</v>
       </c>
       <c r="C17" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="E17" t="s" s="0">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="F17" t="s" s="0">
-        <v>54</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C18" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D18" t="s" s="0">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E18" t="s" s="0">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="F18" t="s" s="0">
-        <v>19</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="C19" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D19" t="s" s="0">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="E19" t="s" s="0">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="F19" t="s" s="0">
         <v>53</v>
@@ -792,119 +849,119 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C20" t="b" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D20" t="s" s="0">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="E20" t="s" s="0">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="F20" t="s" s="0">
-        <v>64</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B21" t="s" s="0">
         <v>60</v>
-      </c>
-      <c r="B21" t="s" s="0">
-        <v>45</v>
       </c>
       <c r="C21" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="E21" t="s" s="0">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="F21" t="s" s="0">
-        <v>48</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="C22" t="b" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" t="s" s="0">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="E22" t="s" s="0">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="F22" t="s" s="0">
-        <v>48</v>
+        <v>41</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="C23" t="b" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23" t="s" s="0">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="E23" t="s" s="0">
-        <v>67</v>
+        <v>24</v>
       </c>
       <c r="F23" t="s" s="0">
-        <v>48</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C24" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D24" t="s" s="0">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="E24" t="s" s="0">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="F24" t="s" s="0">
-        <v>9</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C25" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D25" t="s" s="0">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E25" t="s" s="0">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="F25" t="s" s="0">
         <v>32</v>
@@ -912,242 +969,242 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>71</v>
+        <v>51</v>
       </c>
       <c r="C26" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D26" t="s" s="0">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="E26" t="s" s="0">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="F26" t="s" s="0">
-        <v>21</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="C27" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D27" t="s" s="0">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E27" t="s" s="0">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F27" t="s" s="0">
-        <v>21</v>
+        <v>69</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C28" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D28" t="s" s="0">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="E28" t="s" s="0">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="F28" t="s" s="0">
-        <v>76</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C29" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="E29" t="s" s="0">
-        <v>18</v>
+        <v>74</v>
       </c>
       <c r="F29" t="s" s="0">
-        <v>19</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="C30" t="b" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D30" t="s" s="0">
-        <v>79</v>
+        <v>56</v>
       </c>
       <c r="E30" t="s" s="0">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F30" t="s" s="0">
-        <v>23</v>
+        <v>58</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="C31" t="b" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D31" t="s" s="0">
-        <v>79</v>
+        <v>56</v>
       </c>
       <c r="E31" t="s" s="0">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="F31" t="s" s="0">
-        <v>9</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="B32" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C32" t="b" s="0">
+        <v>0</v>
+      </c>
+      <c r="D32" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="E32" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="F32" t="s" s="0">
         <v>58</v>
-      </c>
-      <c r="C32" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D32" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="E32" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="F32" t="s" s="0">
-        <v>21</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="C33" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D33" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E33" t="s" s="0">
         <v>81</v>
       </c>
-      <c r="B33" t="s" s="0">
-        <v>58</v>
-      </c>
-      <c r="C33" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D33" t="s" s="0">
-        <v>59</v>
-      </c>
-      <c r="E33" t="s" s="0">
-        <v>35</v>
-      </c>
       <c r="F33" t="s" s="0">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C34" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D34" t="s" s="0">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E34" t="s" s="0">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="F34" t="s" s="0">
-        <v>32</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>37</v>
+        <v>83</v>
       </c>
       <c r="C35" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D35" t="s" s="0">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="E35" t="s" s="0">
-        <v>80</v>
+        <v>24</v>
       </c>
       <c r="F35" t="s" s="0">
-        <v>23</v>
+        <v>41</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>86</v>
+        <v>12</v>
       </c>
       <c r="C36" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D36" t="s" s="0">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="E36" t="s" s="0">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F36" t="s" s="0">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C37" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D37" t="s" s="0">
-        <v>79</v>
+        <v>18</v>
       </c>
       <c r="E37" t="s" s="0">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="F37" t="s" s="0">
-        <v>31</v>
+        <v>24</v>
       </c>
     </row>
     <row r="38">
@@ -1161,253 +1218,253 @@
         <v>1</v>
       </c>
       <c r="D38" t="s" s="0">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="E38" t="s" s="0">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F38" t="s" s="0">
-        <v>9</v>
+        <v>26</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C39" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D39" t="s" s="0">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="E39" t="s" s="0">
-        <v>91</v>
+        <v>19</v>
       </c>
       <c r="F39" t="s" s="0">
-        <v>92</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C40" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D40" t="s" s="0">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E40" t="s" s="0">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F40" t="s" s="0">
-        <v>9</v>
+        <v>24</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="C41" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D41" t="s" s="0">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="E41" t="s" s="0">
-        <v>9</v>
+        <v>91</v>
       </c>
       <c r="F41" t="s" s="0">
-        <v>10</v>
+        <v>81</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="C42" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D42" t="s" s="0">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E42" t="s" s="0">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="F42" t="s" s="0">
-        <v>22</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>40</v>
+        <v>93</v>
       </c>
       <c r="C43" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D43" t="s" s="0">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E43" t="s" s="0">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="F43" t="s" s="0">
-        <v>9</v>
+        <v>32</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C44" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D44" t="s" s="0">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="E44" t="s" s="0">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F44" t="s" s="0">
-        <v>32</v>
+        <v>15</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="C45" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D45" t="s" s="0">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="E45" t="s" s="0">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F45" t="s" s="0">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="B46" t="s" s="0">
         <v>97</v>
       </c>
-      <c r="B46" t="s" s="0">
-        <v>37</v>
-      </c>
       <c r="C46" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D46" t="s" s="0">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="E46" t="s" s="0">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F46" t="s" s="0">
-        <v>41</v>
+        <v>19</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="B47" t="s" s="0">
         <v>97</v>
       </c>
-      <c r="B47" t="s" s="0">
-        <v>37</v>
-      </c>
       <c r="C47" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="E47" t="s" s="0">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F47" t="s" s="0">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="C48" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D48" t="s" s="0">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E48" t="s" s="0">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="F48" t="s" s="0">
-        <v>31</v>
+        <v>100</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C49" t="b" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D49" t="s" s="0">
-        <v>46</v>
+        <v>18</v>
       </c>
       <c r="E49" t="s" s="0">
-        <v>100</v>
+        <v>9</v>
       </c>
       <c r="F49" t="s" s="0">
-        <v>48</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C50" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D50" t="s" s="0">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="E50" t="s" s="0">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="F50" t="s" s="0">
-        <v>53</v>
+        <v>104</v>
       </c>
     </row>
     <row r="51">
@@ -1415,219 +1472,219 @@
         <v>102</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="C51" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D51" t="s" s="0">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E51" t="s" s="0">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F51" t="s" s="0">
-        <v>31</v>
+        <v>48</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="C52" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D52" t="s" s="0">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E52" t="s" s="0">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="F52" t="s" s="0">
-        <v>9</v>
+        <v>40</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>37</v>
+        <v>64</v>
       </c>
       <c r="C53" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D53" t="s" s="0">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E53" t="s" s="0">
-        <v>53</v>
+        <v>106</v>
       </c>
       <c r="F53" t="s" s="0">
-        <v>54</v>
+        <v>9</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="0">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>105</v>
+        <v>38</v>
       </c>
       <c r="C54" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D54" t="s" s="0">
-        <v>59</v>
+        <v>8</v>
       </c>
       <c r="E54" t="s" s="0">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="F54" t="s" s="0">
-        <v>32</v>
+        <v>41</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>105</v>
+        <v>38</v>
       </c>
       <c r="C55" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D55" t="s" s="0">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="E55" t="s" s="0">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="F55" t="s" s="0">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B56" t="s" s="0">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="C56" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D56" t="s" s="0">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="E56" t="s" s="0">
-        <v>75</v>
+        <v>14</v>
       </c>
       <c r="F56" t="s" s="0">
-        <v>76</v>
+        <v>15</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="0">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C57" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D57" t="s" s="0">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E57" t="s" s="0">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="F57" t="s" s="0">
-        <v>22</v>
+        <v>48</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="0">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B58" t="s" s="0">
-        <v>108</v>
+        <v>45</v>
       </c>
       <c r="C58" t="b" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D58" t="s" s="0">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="E58" t="s" s="0">
-        <v>109</v>
+        <v>23</v>
       </c>
       <c r="F58" t="s" s="0">
-        <v>48</v>
+        <v>24</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="0">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B59" t="s" s="0">
-        <v>111</v>
+        <v>45</v>
       </c>
       <c r="C59" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D59" t="s" s="0">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="E59" t="s" s="0">
-        <v>41</v>
+        <v>104</v>
       </c>
       <c r="F59" t="s" s="0">
-        <v>42</v>
+        <v>91</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="0">
+        <v>109</v>
+      </c>
+      <c r="B60" t="s" s="0">
         <v>110</v>
       </c>
-      <c r="B60" t="s" s="0">
-        <v>111</v>
-      </c>
       <c r="C60" t="b" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D60" t="s" s="0">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="E60" t="s" s="0">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="F60" t="s" s="0">
-        <v>31</v>
+        <v>58</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="0">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B61" t="s" s="0">
-        <v>82</v>
+        <v>111</v>
       </c>
       <c r="C61" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D61" t="s" s="0">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="E61" t="s" s="0">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="F61" t="s" s="0">
-        <v>21</v>
+        <v>32</v>
       </c>
     </row>
     <row r="62">
@@ -1635,19 +1692,19 @@
         <v>112</v>
       </c>
       <c r="B62" t="s" s="0">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="C62" t="b" s="0">
         <v>1</v>
       </c>
       <c r="D62" t="s" s="0">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="E62" t="s" s="0">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="F62" t="s" s="0">
-        <v>32</v>
+        <v>10</v>
       </c>
     </row>
     <row r="63">
@@ -1655,19 +1712,399 @@
         <v>112</v>
       </c>
       <c r="B63" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="C63" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D63" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E63" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="F63" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s" s="0">
         <v>113</v>
       </c>
-      <c r="C63" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="D63" t="s" s="0">
-        <v>79</v>
-      </c>
-      <c r="E63" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="F63" t="s" s="0">
-        <v>28</v>
+      <c r="B64" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="C64" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D64" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E64" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="F64" t="s" s="0">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="B65" t="s" s="0">
+        <v>115</v>
+      </c>
+      <c r="C65" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D65" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="E65" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F65" t="s" s="0">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s" s="0">
+        <v>118</v>
+      </c>
+      <c r="B66" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C66" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D66" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="E66" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s" s="0">
+        <v>119</v>
+      </c>
+      <c r="B67" t="s" s="0">
+        <v>120</v>
+      </c>
+      <c r="C67" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D67" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="E67" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="F67" t="s" s="0">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s" s="0">
+        <v>119</v>
+      </c>
+      <c r="B68" t="s" s="0">
+        <v>120</v>
+      </c>
+      <c r="C68" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D68" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="E68" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="F68" t="s" s="0">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s" s="0">
+        <v>121</v>
+      </c>
+      <c r="B69" t="s" s="0">
+        <v>111</v>
+      </c>
+      <c r="C69" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D69" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="E69" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="F69" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s" s="0">
+        <v>122</v>
+      </c>
+      <c r="B70" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C70" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D70" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="E70" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="F70" t="s" s="0">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s" s="0">
+        <v>123</v>
+      </c>
+      <c r="B71" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="C71" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D71" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="E71" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F71" t="s" s="0">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s" s="0">
+        <v>123</v>
+      </c>
+      <c r="B72" t="s" s="0">
+        <v>124</v>
+      </c>
+      <c r="C72" t="b" s="0">
+        <v>0</v>
+      </c>
+      <c r="D72" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="E72" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="F72" t="s" s="0">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s" s="0">
+        <v>125</v>
+      </c>
+      <c r="B73" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="C73" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D73" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E73" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="F73" t="s" s="0">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="s" s="0">
+        <v>126</v>
+      </c>
+      <c r="B74" t="s" s="0">
+        <v>127</v>
+      </c>
+      <c r="C74" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D74" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="E74" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="F74" t="s" s="0">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="B75" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="C75" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D75" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="E75" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F75" t="s" s="0">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="B76" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="C76" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D76" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E76" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="F76" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="s" s="0">
+        <v>129</v>
+      </c>
+      <c r="B77" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="C77" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D77" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E77" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="F77" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="s" s="0">
+        <v>129</v>
+      </c>
+      <c r="B78" t="s" s="0">
+        <v>130</v>
+      </c>
+      <c r="C78" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D78" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="E78" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="F78" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s" s="0">
+        <v>129</v>
+      </c>
+      <c r="B79" t="s" s="0">
+        <v>130</v>
+      </c>
+      <c r="C79" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D79" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E79" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="F79" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s" s="0">
+        <v>131</v>
+      </c>
+      <c r="B80" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C80" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D80" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E80" t="s" s="0">
+        <v>117</v>
+      </c>
+      <c r="F80" t="s" s="0">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="s" s="0">
+        <v>131</v>
+      </c>
+      <c r="B81" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C81" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D81" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="E81" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="F81" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="s" s="0">
+        <v>131</v>
+      </c>
+      <c r="B82" t="s" s="0">
+        <v>111</v>
+      </c>
+      <c r="C82" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D82" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E82" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="F82" t="s" s="0">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: updated Schedule config to be used as a singleton class
</commit_message>
<xml_diff>
--- a/java/hello-world/src/main/java/org/acme/schooltimetabling/generated/temp.xlsx
+++ b/java/hello-world/src/main/java/org/acme/schooltimetabling/generated/temp.xlsx
@@ -48,492 +48,501 @@
     <t>1</t>
   </si>
   <si>
+    <t>232A</t>
+  </si>
+  <si>
+    <t>MWF 09:00 - 10:00</t>
+  </si>
+  <si>
+    <t>MWF 10:00 - 11:00</t>
+  </si>
+  <si>
+    <t>Stephen Beard</t>
+  </si>
+  <si>
+    <t>csc430</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>TR 08:00 - 09:30</t>
+  </si>
+  <si>
+    <t>TR 09:30 - 11:00</t>
+  </si>
+  <si>
+    <t>John Bellardo</t>
+  </si>
+  <si>
+    <t>csc454</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
     <t>301</t>
   </si>
   <si>
+    <t>TR 15:00 - 16:30</t>
+  </si>
+  <si>
+    <t>TR 16:30 - 18:00</t>
+  </si>
+  <si>
+    <t>John Clements</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>302</t>
+  </si>
+  <si>
+    <t>MWF 15:00 - 16:00</t>
+  </si>
+  <si>
+    <t>MWF 16:00 - 17:00</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Rodrigo Canaan</t>
+  </si>
+  <si>
+    <t>csc480</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>MWF 07:00 - 08:00</t>
+  </si>
+  <si>
     <t>MWF 08:00 - 09:00</t>
   </si>
   <si>
-    <t>MWF 09:00 - 10:00</t>
-  </si>
-  <si>
-    <t>Stephen Beard</t>
-  </si>
-  <si>
-    <t>csc430</t>
-  </si>
-  <si>
-    <t>2</t>
+    <t>csc481</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>192-206</t>
+  </si>
+  <si>
+    <t>TR 16:00 - 17:30</t>
+  </si>
+  <si>
+    <t>TR 17:30 - 19:00</t>
+  </si>
+  <si>
+    <t>Alex Dekhtyar</t>
+  </si>
+  <si>
+    <t>csc365</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>255</t>
+  </si>
+  <si>
+    <t>Duran, Kirk Alberto</t>
+  </si>
+  <si>
+    <t>csc101</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>MWF 19:00 - 20:00</t>
+  </si>
+  <si>
+    <t>MWF 20:00 - 21:00</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>MWF 17:00 - 18:00</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>TR 19:00 - 20:30</t>
+  </si>
+  <si>
+    <t>TR 20:30 - 22:00</t>
+  </si>
+  <si>
+    <t>Christian Eckhardt</t>
+  </si>
+  <si>
+    <t>csc357</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>csc474</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>TR 12:00 - 13:30</t>
+  </si>
+  <si>
+    <t>TR 13:30 - 15:00</t>
+  </si>
+  <si>
+    <t>Sussan Einakian</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>MWF 13:00 - 14:00</t>
+  </si>
+  <si>
+    <t>MWF 14:00 - 15:00</t>
+  </si>
+  <si>
+    <t>Fang, Dongfeng</t>
+  </si>
+  <si>
+    <t>csc321</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>18</t>
   </si>
   <si>
     <t>192-333</t>
   </si>
   <si>
-    <t>TR 08:00 - 09:30</t>
-  </si>
-  <si>
-    <t>TR 09:30 - 11:00</t>
-  </si>
-  <si>
-    <t>John Bellardo</t>
-  </si>
-  <si>
-    <t>csc454</t>
-  </si>
-  <si>
-    <t>3</t>
+    <t>MWF 18:00 - 19:00</t>
+  </si>
+  <si>
+    <t>Daniel Frishberg</t>
+  </si>
+  <si>
+    <t>csc445</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>LECTURE_ONLY</t>
+  </si>
+  <si>
+    <t>MTWR 15:00 - 16:00</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Javier Gonzalez Sanchez</t>
+  </si>
+  <si>
+    <t>csc570</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>MTWR 17:00 - 18:00</t>
+  </si>
+  <si>
+    <t>April Grow</t>
+  </si>
+  <si>
+    <t>csc378</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>TR 17:00 - 18:30</t>
+  </si>
+  <si>
+    <t>TR 18:30 - 20:00</t>
+  </si>
+  <si>
+    <t>Han, Wei-jer</t>
+  </si>
+  <si>
+    <t>csc225</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>256</t>
+  </si>
+  <si>
+    <t>Hartman, Bret Andrew</t>
+  </si>
+  <si>
+    <t>csc422</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>Borislav Hristov</t>
+  </si>
+  <si>
+    <t>csc448</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>Silas Hsu</t>
+  </si>
+  <si>
+    <t>csc437</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>TR 20:00 - 21:30</t>
+  </si>
+  <si>
+    <t>Brian Jones</t>
+  </si>
+  <si>
+    <t>csc232</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>TR 17:00 - 18:00</t>
+  </si>
+  <si>
+    <t>TR 18:00 - 19:00</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>MTWR 19:00 - 20:00</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>MTWR 16:00 - 17:00</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>Paris Kalathas</t>
+  </si>
+  <si>
+    <t>csc203</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>Ayaan Kazerouni</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>MWF 11:00 - 12:00</t>
+  </si>
+  <si>
+    <t>csc477</t>
+  </si>
+  <si>
+    <t>34</t>
   </si>
   <si>
     <t>257</t>
   </si>
   <si>
-    <t>TR 15:00 - 16:30</t>
-  </si>
-  <si>
-    <t>TR 16:30 - 18:00</t>
-  </si>
-  <si>
-    <t>John Clements</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>192-206</t>
-  </si>
-  <si>
-    <t>MWF 15:00 - 16:00</t>
-  </si>
-  <si>
-    <t>MWF 16:00 - 17:00</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>TR 12:00 - 13:30</t>
-  </si>
-  <si>
-    <t>TR 13:30 - 15:00</t>
-  </si>
-  <si>
-    <t>Rodrigo Canaan</t>
-  </si>
-  <si>
-    <t>csc480</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>302</t>
+    <t>Aaron Keen</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>Fahim Khan</t>
+  </si>
+  <si>
+    <t>csc471</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>BJ Klingenberg</t>
+  </si>
+  <si>
+    <t>csc406</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>Ken Kubiak</t>
+  </si>
+  <si>
+    <t>csc307</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>MWF 12:00 - 13:00</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>41</t>
+  </si>
+  <si>
+    <t>Ulf Lindqvist</t>
+  </si>
+  <si>
+    <t>csc320</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>Joydeep Mukherjee</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
+    <t>csc410</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>Phillip Nico</t>
+  </si>
+  <si>
+    <t>csc453</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>46</t>
+  </si>
+  <si>
+    <t>Maria Pantoja</t>
+  </si>
+  <si>
+    <t>csc569</t>
+  </si>
+  <si>
+    <t>47</t>
+  </si>
+  <si>
+    <t>Zachary Peterson</t>
+  </si>
+  <si>
+    <t>48</t>
+  </si>
+  <si>
+    <t>Lucas Pierce</t>
+  </si>
+  <si>
+    <t>csc466</t>
+  </si>
+  <si>
+    <t>49</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>Planck, John R.</t>
+  </si>
+  <si>
+    <t>51</t>
   </si>
   <si>
     <t>TR 18:00 - 19:30</t>
   </si>
   <si>
-    <t>csc481</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>MWF 18:00 - 19:00</t>
-  </si>
-  <si>
-    <t>MWF 19:00 - 20:00</t>
-  </si>
-  <si>
-    <t>Alex Dekhtyar</t>
-  </si>
-  <si>
-    <t>csc365</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>Duran, Kirk Alberto</t>
-  </si>
-  <si>
-    <t>csc101</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>232A</t>
-  </si>
-  <si>
-    <t>MWF 17:00 - 18:00</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>MWF 07:00 - 08:00</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>Christian Eckhardt</t>
-  </si>
-  <si>
-    <t>csc357</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>csc474</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>255</t>
-  </si>
-  <si>
-    <t>Sussan Einakian</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>MWF 10:00 - 11:00</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>MWF 13:00 - 14:00</t>
-  </si>
-  <si>
-    <t>MWF 14:00 - 15:00</t>
-  </si>
-  <si>
-    <t>Fang, Dongfeng</t>
-  </si>
-  <si>
-    <t>csc321</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>TR 19:00 - 20:30</t>
-  </si>
-  <si>
-    <t>TR 20:30 - 22:00</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>Daniel Frishberg</t>
-  </si>
-  <si>
-    <t>csc445</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>LECTURE_ONLY</t>
-  </si>
-  <si>
-    <t>MTWR 15:00 - 16:00</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Javier Gonzalez Sanchez</t>
-  </si>
-  <si>
-    <t>csc570</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>MTWR 16:00 - 17:00</t>
-  </si>
-  <si>
-    <t>April Grow</t>
-  </si>
-  <si>
-    <t>csc378</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>Han, Wei-jer</t>
-  </si>
-  <si>
-    <t>csc225</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>MWF 20:00 - 21:00</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>Hartman, Bret Andrew</t>
-  </si>
-  <si>
-    <t>csc422</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>Borislav Hristov</t>
-  </si>
-  <si>
-    <t>csc448</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>Silas Hsu</t>
-  </si>
-  <si>
-    <t>csc437</t>
-  </si>
-  <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>Brian Jones</t>
-  </si>
-  <si>
-    <t>csc232</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>TR 15:00 - 16:00</t>
-  </si>
-  <si>
-    <t>TR 16:00 - 17:00</t>
-  </si>
-  <si>
-    <t>29</t>
-  </si>
-  <si>
-    <t>MTWR 17:00 - 18:00</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>MTWR 19:00 - 20:00</t>
-  </si>
-  <si>
-    <t>31</t>
+    <t>TR 19:30 - 21:00</t>
+  </si>
+  <si>
+    <t>52</t>
+  </si>
+  <si>
+    <t>Anita Rathi</t>
+  </si>
+  <si>
+    <t>53</t>
+  </si>
+  <si>
+    <t>54</t>
+  </si>
+  <si>
+    <t>55</t>
+  </si>
+  <si>
+    <t>Vanessa Rivera</t>
+  </si>
+  <si>
+    <t>56</t>
+  </si>
+  <si>
+    <t>57</t>
+  </si>
+  <si>
+    <t>58</t>
+  </si>
+  <si>
+    <t>Mugizi Rwebangira</t>
+  </si>
+  <si>
+    <t>csc566</t>
+  </si>
+  <si>
+    <t>59</t>
   </si>
   <si>
     <t>MTWR 18:00 - 19:00</t>
   </si>
   <si>
-    <t>Paris Kalathas</t>
-  </si>
-  <si>
-    <t>csc203</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>Ayaan Kazerouni</t>
-  </si>
-  <si>
-    <t>33</t>
-  </si>
-  <si>
-    <t>csc477</t>
-  </si>
-  <si>
-    <t>34</t>
-  </si>
-  <si>
-    <t>MWF 11:00 - 12:00</t>
-  </si>
-  <si>
-    <t>Aaron Keen</t>
-  </si>
-  <si>
-    <t>35</t>
-  </si>
-  <si>
-    <t>Fahim Khan</t>
-  </si>
-  <si>
-    <t>csc471</t>
-  </si>
-  <si>
-    <t>36</t>
-  </si>
-  <si>
-    <t>BJ Klingenberg</t>
-  </si>
-  <si>
-    <t>csc406</t>
-  </si>
-  <si>
-    <t>37</t>
-  </si>
-  <si>
-    <t>256</t>
-  </si>
-  <si>
-    <t>38</t>
-  </si>
-  <si>
-    <t>Ken Kubiak</t>
-  </si>
-  <si>
-    <t>csc307</t>
-  </si>
-  <si>
-    <t>39</t>
-  </si>
-  <si>
-    <t>40</t>
-  </si>
-  <si>
-    <t>41</t>
-  </si>
-  <si>
-    <t>Ulf Lindqvist</t>
-  </si>
-  <si>
-    <t>csc320</t>
-  </si>
-  <si>
-    <t>42</t>
-  </si>
-  <si>
-    <t>Joydeep Mukherjee</t>
-  </si>
-  <si>
-    <t>43</t>
-  </si>
-  <si>
-    <t>csc410</t>
-  </si>
-  <si>
-    <t>44</t>
-  </si>
-  <si>
-    <t>Phillip Nico</t>
-  </si>
-  <si>
-    <t>csc453</t>
-  </si>
-  <si>
-    <t>45</t>
-  </si>
-  <si>
-    <t>46</t>
-  </si>
-  <si>
-    <t>Maria Pantoja</t>
-  </si>
-  <si>
-    <t>csc569</t>
-  </si>
-  <si>
-    <t>47</t>
-  </si>
-  <si>
-    <t>TR 17:00 - 18:30</t>
-  </si>
-  <si>
-    <t>TR 18:30 - 20:00</t>
-  </si>
-  <si>
-    <t>Zachary Peterson</t>
-  </si>
-  <si>
-    <t>48</t>
-  </si>
-  <si>
-    <t>Lucas Pierce</t>
-  </si>
-  <si>
-    <t>csc466</t>
-  </si>
-  <si>
-    <t>49</t>
-  </si>
-  <si>
-    <t>MWF 12:00 - 13:00</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t>Planck, John R.</t>
-  </si>
-  <si>
-    <t>51</t>
-  </si>
-  <si>
-    <t>52</t>
-  </si>
-  <si>
-    <t>Anita Rathi</t>
-  </si>
-  <si>
-    <t>53</t>
-  </si>
-  <si>
-    <t>54</t>
-  </si>
-  <si>
-    <t>55</t>
-  </si>
-  <si>
-    <t>Vanessa Rivera</t>
-  </si>
-  <si>
-    <t>56</t>
-  </si>
-  <si>
-    <t>57</t>
-  </si>
-  <si>
-    <t>58</t>
-  </si>
-  <si>
-    <t>Mugizi Rwebangira</t>
-  </si>
-  <si>
-    <t>csc566</t>
-  </si>
-  <si>
-    <t>59</t>
-  </si>
-  <si>
-    <t>TR 16:00 - 18:00</t>
-  </si>
-  <si>
     <t>csc349</t>
   </si>
   <si>
@@ -564,9 +573,6 @@
     <t>64</t>
   </si>
   <si>
-    <t>TR 17:30 - 19:00</t>
-  </si>
-  <si>
     <t>Christopher Siu</t>
   </si>
   <si>
@@ -591,9 +597,6 @@
     <t>68</t>
   </si>
   <si>
-    <t>TR 16:00 - 17:30</t>
-  </si>
-  <si>
     <t>Vargas, Luis E.</t>
   </si>
   <si>
@@ -625,9 +628,6 @@
   </si>
   <si>
     <t>73</t>
-  </si>
-  <si>
-    <t>TR 20:00 - 21:30</t>
   </si>
   <si>
     <t>Eric Yocam</t>
@@ -784,1565 +784,1565 @@
         <v>1</v>
       </c>
       <c r="F3" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s" s="0">
         <v>17</v>
       </c>
-      <c r="G3" t="s" s="0">
+      <c r="H3" t="s" s="0">
         <v>18</v>
-      </c>
-      <c r="H3" t="s" s="0">
-        <v>19</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s" s="0">
         <v>20</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="C4" t="s" s="0">
         <v>21</v>
       </c>
-      <c r="C4" t="s" s="0">
+      <c r="E4" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="E4" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="F4" t="s" s="0">
+      <c r="G4" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="G4" t="s" s="0">
+      <c r="H4" t="s" s="0">
         <v>24</v>
-      </c>
-      <c r="H4" t="s" s="0">
-        <v>25</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s" s="0">
         <v>15</v>
       </c>
       <c r="C5" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="E5" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s" s="0">
         <v>27</v>
       </c>
-      <c r="E5" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="F5" t="s" s="0">
+      <c r="G5" t="s" s="0">
         <v>28</v>
       </c>
-      <c r="G5" t="s" s="0">
+      <c r="H5" t="s" s="0">
         <v>29</v>
-      </c>
-      <c r="H5" t="s" s="0">
-        <v>30</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>9</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E6" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>33</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E7" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="G7" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="H7" t="s" s="0">
         <v>35</v>
-      </c>
-      <c r="C7" t="s" s="0">
-        <v>36</v>
-      </c>
-      <c r="E7" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="F7" t="s" s="0">
-        <v>37</v>
-      </c>
-      <c r="G7" t="s" s="0">
-        <v>25</v>
-      </c>
-      <c r="H7" t="s" s="0">
-        <v>38</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B8" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="E8" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="G8" t="s" s="0">
         <v>39</v>
       </c>
-      <c r="C8" t="s" s="0">
+      <c r="H8" t="s" s="0">
         <v>40</v>
-      </c>
-      <c r="E8" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="F8" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="G8" t="s" s="0">
-        <v>41</v>
-      </c>
-      <c r="H8" t="s" s="0">
-        <v>42</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C9" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="B9" t="s" s="0">
+      <c r="E9" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="F9" t="s" s="0">
         <v>44</v>
       </c>
-      <c r="C9" t="s" s="0">
-        <v>45</v>
-      </c>
-      <c r="E9" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="F9" t="s" s="0">
-        <v>17</v>
-      </c>
       <c r="G9" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="H9" t="s" s="0">
         <v>29</v>
-      </c>
-      <c r="H9" t="s" s="0">
-        <v>30</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="B10" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="B10" t="s" s="0">
+      <c r="C10" t="s" s="0">
         <v>47</v>
       </c>
-      <c r="C10" t="s" s="0">
+      <c r="E10" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="G10" t="s" s="0">
         <v>48</v>
       </c>
-      <c r="E10" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="F10" t="s" s="0">
+      <c r="H10" t="s" s="0">
         <v>49</v>
-      </c>
-      <c r="G10" t="s" s="0">
-        <v>30</v>
-      </c>
-      <c r="H10" t="s" s="0">
-        <v>50</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="B11" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="B11" t="s" s="0">
-        <v>47</v>
-      </c>
       <c r="C11" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="E11" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="F11" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="G11" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="H11" t="s" s="0">
         <v>51</v>
-      </c>
-      <c r="E11" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="F11" t="s" s="0">
-        <v>49</v>
-      </c>
-      <c r="G11" t="s" s="0">
-        <v>52</v>
-      </c>
-      <c r="H11" t="s" s="0">
-        <v>12</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B12" t="s" s="0">
         <v>9</v>
       </c>
       <c r="C12" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E12" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="G12" t="s" s="0">
         <v>53</v>
       </c>
-      <c r="E12" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="F12" t="s" s="0">
-        <v>49</v>
-      </c>
-      <c r="G12" t="s" s="0">
-        <v>25</v>
-      </c>
       <c r="H12" t="s" s="0">
-        <v>38</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E13" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="G13" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="H13" t="s" s="0">
         <v>24</v>
-      </c>
-      <c r="H13" t="s" s="0">
-        <v>25</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E14" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F14" t="s" s="0">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="G14" t="s" s="0">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="H14" t="s" s="0">
-        <v>19</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C15" t="s" s="0">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E15" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F15" t="s" s="0">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="G15" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="H15" t="s" s="0">
         <v>29</v>
-      </c>
-      <c r="H15" t="s" s="0">
-        <v>30</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B16" t="s" s="0">
         <v>9</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E16" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F16" t="s" s="0">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="G16" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="H16" t="s" s="0">
         <v>13</v>
-      </c>
-      <c r="H16" t="s" s="0">
-        <v>63</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B17" t="s" s="0">
         <v>9</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E17" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F17" t="s" s="0">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="G17" t="s" s="0">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H17" t="s" s="0">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C18" t="s" s="0">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E18" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F18" t="s" s="0">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="G18" t="s" s="0">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="H18" t="s" s="0">
-        <v>71</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C19" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="E19" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="F19" t="s" s="0">
         <v>72</v>
       </c>
-      <c r="E19" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="F19" t="s" s="0">
-        <v>28</v>
-      </c>
       <c r="G19" t="s" s="0">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="H19" t="s" s="0">
-        <v>25</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C20" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E20" t="b" s="0">
         <v>0</v>
       </c>
       <c r="F20" t="s" s="0">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G20" t="s" s="0">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H20" t="s" s="0">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C21" t="s" s="0">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E21" t="b" s="0">
         <v>0</v>
       </c>
       <c r="F21" t="s" s="0">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G21" t="s" s="0">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H21" t="s" s="0">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C22" t="s" s="0">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E22" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F22" t="s" s="0">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="G22" t="s" s="0">
-        <v>30</v>
+        <v>87</v>
       </c>
       <c r="H22" t="s" s="0">
-        <v>50</v>
+        <v>88</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C23" t="s" s="0">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E23" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F23" t="s" s="0">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="G23" t="s" s="0">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="H23" t="s" s="0">
-        <v>89</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C24" t="s" s="0">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E24" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F24" t="s" s="0">
-        <v>59</v>
+        <v>93</v>
       </c>
       <c r="G24" t="s" s="0">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H24" t="s" s="0">
-        <v>12</v>
+        <v>73</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C25" t="s" s="0">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E25" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F25" t="s" s="0">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="G25" t="s" s="0">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H25" t="s" s="0">
-        <v>41</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C26" t="s" s="0">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E26" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F26" t="s" s="0">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G26" t="s" s="0">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="H26" t="s" s="0">
-        <v>89</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C27" t="s" s="0">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="E27" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F27" t="s" s="0">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="G27" t="s" s="0">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="H27" t="s" s="0">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C28" t="s" s="0">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="E28" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F28" t="s" s="0">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="G28" t="s" s="0">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="H28" t="s" s="0">
-        <v>89</v>
+        <v>104</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C29" t="s" s="0">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="E29" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F29" t="s" s="0">
-        <v>59</v>
+        <v>93</v>
       </c>
       <c r="G29" t="s" s="0">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="H29" t="s" s="0">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C30" t="s" s="0">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E30" t="b" s="0">
         <v>0</v>
       </c>
       <c r="F30" t="s" s="0">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G30" t="s" s="0">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="H30" t="s" s="0">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C31" t="s" s="0">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E31" t="b" s="0">
         <v>0</v>
       </c>
       <c r="F31" t="s" s="0">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G31" t="s" s="0">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H31" t="s" s="0">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C32" t="s" s="0">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E32" t="b" s="0">
         <v>0</v>
       </c>
       <c r="F32" t="s" s="0">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G32" t="s" s="0">
-        <v>111</v>
+        <v>78</v>
       </c>
       <c r="H32" t="s" s="0">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C33" t="s" s="0">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="E33" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F33" t="s" s="0">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="G33" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="H33" t="s" s="0">
         <v>12</v>
-      </c>
-      <c r="H33" t="s" s="0">
-        <v>13</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C34" t="s" s="0">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E34" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F34" t="s" s="0">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="G34" t="s" s="0">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="H34" t="s" s="0">
-        <v>50</v>
+        <v>120</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C35" t="s" s="0">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E35" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F35" t="s" s="0">
-        <v>49</v>
+        <v>123</v>
       </c>
       <c r="G35" t="s" s="0">
-        <v>63</v>
+        <v>29</v>
       </c>
       <c r="H35" t="s" s="0">
-        <v>119</v>
+        <v>51</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B36" t="s" s="0">
         <v>15</v>
       </c>
       <c r="C36" t="s" s="0">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="E36" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F36" t="s" s="0">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="G36" t="s" s="0">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="H36" t="s" s="0">
-        <v>119</v>
+        <v>12</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C37" t="s" s="0">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="E37" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F37" t="s" s="0">
-        <v>59</v>
+        <v>93</v>
       </c>
       <c r="G37" t="s" s="0">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="H37" t="s" s="0">
-        <v>41</v>
+        <v>48</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C38" t="s" s="0">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="E38" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F38" t="s" s="0">
-        <v>128</v>
+        <v>93</v>
       </c>
       <c r="G38" t="s" s="0">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="H38" t="s" s="0">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C39" t="s" s="0">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E39" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F39" t="s" s="0">
-        <v>128</v>
+        <v>93</v>
       </c>
       <c r="G39" t="s" s="0">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="H39" t="s" s="0">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C40" t="s" s="0">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E40" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F40" t="s" s="0">
-        <v>128</v>
+        <v>93</v>
       </c>
       <c r="G40" t="s" s="0">
-        <v>33</v>
+        <v>136</v>
       </c>
       <c r="H40" t="s" s="0">
-        <v>24</v>
+        <v>66</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C41" t="s" s="0">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="E41" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F41" t="s" s="0">
-        <v>128</v>
+        <v>38</v>
       </c>
       <c r="G41" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="H41" t="s" s="0">
         <v>12</v>
-      </c>
-      <c r="H41" t="s" s="0">
-        <v>13</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C42" t="s" s="0">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E42" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F42" t="s" s="0">
-        <v>59</v>
+        <v>123</v>
       </c>
       <c r="G42" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="H42" t="s" s="0">
         <v>29</v>
-      </c>
-      <c r="H42" t="s" s="0">
-        <v>30</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C43" t="s" s="0">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="E43" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F43" t="s" s="0">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G43" t="s" s="0">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="H43" t="s" s="0">
-        <v>50</v>
+        <v>73</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C44" t="s" s="0">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E44" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F44" t="s" s="0">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="G44" t="s" s="0">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="H44" t="s" s="0">
-        <v>33</v>
+        <v>61</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C45" t="s" s="0">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E45" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F45" t="s" s="0">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G45" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="H45" t="s" s="0">
         <v>18</v>
-      </c>
-      <c r="H45" t="s" s="0">
-        <v>19</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C46" t="s" s="0">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="E46" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F46" t="s" s="0">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="G46" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="H46" t="s" s="0">
         <v>12</v>
-      </c>
-      <c r="H46" t="s" s="0">
-        <v>13</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C47" t="s" s="0">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="E47" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F47" t="s" s="0">
-        <v>128</v>
+        <v>72</v>
       </c>
       <c r="G47" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="H47" t="s" s="0">
         <v>29</v>
-      </c>
-      <c r="H47" t="s" s="0">
-        <v>30</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C48" t="s" s="0">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E48" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F48" t="s" s="0">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="G48" t="s" s="0">
-        <v>149</v>
+        <v>40</v>
       </c>
       <c r="H48" t="s" s="0">
-        <v>150</v>
+        <v>53</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C49" t="s" s="0">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E49" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F49" t="s" s="0">
-        <v>23</v>
+        <v>93</v>
       </c>
       <c r="G49" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="H49" t="s" s="0">
         <v>12</v>
-      </c>
-      <c r="H49" t="s" s="0">
-        <v>13</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C50" t="s" s="0">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E50" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F50" t="s" s="0">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="G50" t="s" s="0">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="H50" t="s" s="0">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C51" t="s" s="0">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E51" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F51" t="s" s="0">
-        <v>23</v>
+        <v>93</v>
       </c>
       <c r="G51" t="s" s="0">
-        <v>63</v>
+        <v>12</v>
       </c>
       <c r="H51" t="s" s="0">
-        <v>119</v>
+        <v>13</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C52" t="s" s="0">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E52" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F52" t="s" s="0">
-        <v>11</v>
+        <v>72</v>
       </c>
       <c r="G52" t="s" s="0">
-        <v>52</v>
+        <v>161</v>
       </c>
       <c r="H52" t="s" s="0">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C53" t="s" s="0">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="E53" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F53" t="s" s="0">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="G53" t="s" s="0">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="H53" t="s" s="0">
-        <v>89</v>
+        <v>24</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="0">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C54" t="s" s="0">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E54" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F54" t="s" s="0">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="G54" t="s" s="0">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H54" t="s" s="0">
-        <v>50</v>
+        <v>12</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C55" t="s" s="0">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E55" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F55" t="s" s="0">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="G55" t="s" s="0">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="H55" t="s" s="0">
-        <v>13</v>
+        <v>51</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B56" t="s" s="0">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C56" t="s" s="0">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="E56" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F56" t="s" s="0">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="G56" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="H56" t="s" s="0">
         <v>18</v>
-      </c>
-      <c r="H56" t="s" s="0">
-        <v>19</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="0">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C57" t="s" s="0">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="E57" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F57" t="s" s="0">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="G57" t="s" s="0">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="H57" t="s" s="0">
-        <v>30</v>
+        <v>12</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="0">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B58" t="s" s="0">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C58" t="s" s="0">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="E58" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F58" t="s" s="0">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="G58" t="s" s="0">
-        <v>156</v>
+        <v>28</v>
       </c>
       <c r="H58" t="s" s="0">
-        <v>65</v>
+        <v>29</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="0">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B59" t="s" s="0">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C59" t="s" s="0">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E59" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F59" t="s" s="0">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="G59" t="s" s="0">
         <v>13</v>
       </c>
       <c r="H59" t="s" s="0">
-        <v>63</v>
+        <v>120</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="0">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B60" t="s" s="0">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C60" t="s" s="0">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="E60" t="b" s="0">
         <v>0</v>
       </c>
       <c r="F60" t="s" s="0">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G60" t="s" s="0">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="H60" t="s" s="0">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="0">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B61" t="s" s="0">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C61" t="s" s="0">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="E61" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F61" t="s" s="0">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="G61" t="s" s="0">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="H61" t="s" s="0">
-        <v>41</v>
+        <v>51</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s" s="0">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B62" t="s" s="0">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C62" t="s" s="0">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="E62" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F62" t="s" s="0">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="G62" t="s" s="0">
-        <v>12</v>
+        <v>67</v>
       </c>
       <c r="H62" t="s" s="0">
-        <v>13</v>
+        <v>28</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="0">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B63" t="s" s="0">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C63" t="s" s="0">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="E63" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F63" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G63" t="s" s="0">
-        <v>29</v>
+        <v>120</v>
       </c>
       <c r="H63" t="s" s="0">
-        <v>30</v>
+        <v>136</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s" s="0">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B64" t="s" s="0">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C64" t="s" s="0">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="E64" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F64" t="s" s="0">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="G64" t="s" s="0">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="H64" t="s" s="0">
-        <v>89</v>
+        <v>120</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s" s="0">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B65" t="s" s="0">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C65" t="s" s="0">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="E65" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F65" t="s" s="0">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="G65" t="s" s="0">
-        <v>183</v>
+        <v>51</v>
       </c>
       <c r="H65" t="s" s="0">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s" s="0">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B66" t="s" s="0">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C66" t="s" s="0">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E66" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F66" t="s" s="0">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="G66" t="s" s="0">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="H66" t="s" s="0">
-        <v>30</v>
+        <v>161</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s" s="0">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B67" t="s" s="0">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C67" t="s" s="0">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E67" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F67" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G67" t="s" s="0">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="H67" t="s" s="0">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s" s="0">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B68" t="s" s="0">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C68" t="s" s="0">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E68" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F68" t="s" s="0">
-        <v>128</v>
+        <v>72</v>
       </c>
       <c r="G68" t="s" s="0">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="H68" t="s" s="0">
-        <v>50</v>
+        <v>24</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s" s="0">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B69" t="s" s="0">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C69" t="s" s="0">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E69" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F69" t="s" s="0">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="G69" t="s" s="0">
-        <v>192</v>
+        <v>23</v>
       </c>
       <c r="H69" t="s" s="0">
-        <v>183</v>
+        <v>24</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s" s="0">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B70" t="s" s="0">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C70" t="s" s="0">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E70" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F70" t="s" s="0">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="G70" t="s" s="0">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="H70" t="s" s="0">
-        <v>71</v>
+        <v>48</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s" s="0">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B71" t="s" s="0">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C71" t="s" s="0">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E71" t="b" s="0">
         <v>1</v>
@@ -2351,79 +2351,79 @@
         <v>11</v>
       </c>
       <c r="G71" t="s" s="0">
-        <v>119</v>
+        <v>60</v>
       </c>
       <c r="H71" t="s" s="0">
-        <v>156</v>
+        <v>61</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s" s="0">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B72" t="s" s="0">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C72" t="s" s="0">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E72" t="b" s="0">
         <v>0</v>
       </c>
       <c r="F72" t="s" s="0">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G72" t="s" s="0">
-        <v>77</v>
+        <v>113</v>
       </c>
       <c r="H72" t="s" s="0">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s" s="0">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B73" t="s" s="0">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C73" t="s" s="0">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E73" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F73" t="s" s="0">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="G73" t="s" s="0">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="H73" t="s" s="0">
-        <v>41</v>
+        <v>48</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s" s="0">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B74" t="s" s="0">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C74" t="s" s="0">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E74" t="b" s="0">
         <v>1</v>
       </c>
       <c r="F74" t="s" s="0">
-        <v>23</v>
+        <v>123</v>
       </c>
       <c r="G74" t="s" s="0">
-        <v>150</v>
+        <v>48</v>
       </c>
       <c r="H74" t="s" s="0">
-        <v>204</v>
+        <v>49</v>
       </c>
     </row>
     <row r="75">
@@ -2431,7 +2431,7 @@
         <v>205</v>
       </c>
       <c r="B75" t="s" s="0">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C75" t="s" s="0">
         <v>206</v>
@@ -2440,13 +2440,13 @@
         <v>1</v>
       </c>
       <c r="F75" t="s" s="0">
-        <v>28</v>
+        <v>72</v>
       </c>
       <c r="G75" t="s" s="0">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="H75" t="s" s="0">
-        <v>66</v>
+        <v>13</v>
       </c>
     </row>
     <row r="76">
@@ -2454,7 +2454,7 @@
         <v>205</v>
       </c>
       <c r="B76" t="s" s="0">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C76" t="s" s="0">
         <v>207</v>
@@ -2463,13 +2463,13 @@
         <v>1</v>
       </c>
       <c r="F76" t="s" s="0">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="G76" t="s" s="0">
-        <v>63</v>
+        <v>28</v>
       </c>
       <c r="H76" t="s" s="0">
-        <v>119</v>
+        <v>29</v>
       </c>
     </row>
     <row r="77">
@@ -2477,7 +2477,7 @@
         <v>208</v>
       </c>
       <c r="B77" t="s" s="0">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C77" t="s" s="0">
         <v>209</v>
@@ -2486,13 +2486,13 @@
         <v>1</v>
       </c>
       <c r="F77" t="s" s="0">
-        <v>128</v>
+        <v>93</v>
       </c>
       <c r="G77" t="s" s="0">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H77" t="s" s="0">
-        <v>33</v>
+        <v>51</v>
       </c>
     </row>
     <row r="78">
@@ -2509,13 +2509,13 @@
         <v>1</v>
       </c>
       <c r="F78" t="s" s="0">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G78" t="s" s="0">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="H78" t="s" s="0">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="79">
@@ -2532,13 +2532,13 @@
         <v>1</v>
       </c>
       <c r="F79" t="s" s="0">
-        <v>23</v>
+        <v>93</v>
       </c>
       <c r="G79" t="s" s="0">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="H79" t="s" s="0">
-        <v>50</v>
+        <v>35</v>
       </c>
     </row>
     <row r="80">
@@ -2555,13 +2555,13 @@
         <v>1</v>
       </c>
       <c r="F80" t="s" s="0">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="G80" t="s" s="0">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="H80" t="s" s="0">
-        <v>89</v>
+        <v>49</v>
       </c>
     </row>
     <row r="81">
@@ -2578,13 +2578,13 @@
         <v>1</v>
       </c>
       <c r="F81" t="s" s="0">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="G81" t="s" s="0">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="H81" t="s" s="0">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="82">
@@ -2592,7 +2592,7 @@
         <v>213</v>
       </c>
       <c r="B82" t="s" s="0">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C82" t="s" s="0">
         <v>216</v>
@@ -2601,13 +2601,13 @@
         <v>1</v>
       </c>
       <c r="F82" t="s" s="0">
-        <v>11</v>
+        <v>123</v>
       </c>
       <c r="G82" t="s" s="0">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="H82" t="s" s="0">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>